<commit_message>
Keep type as delivery/discovery and mark vacation separately.
Drop ЦКО from the type list and Отпуск from the role list. Vacation is
a dedicated да column on the real role, so those days are non-working
for that person instead of a fake specialty.

Co-authored-by: bbenicore-web <bbenicore-web@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/templates/Календаризация_шаблон.xlsx
+++ b/templates/Календаризация_шаблон.xlsx
@@ -12,7 +12,7 @@
     <sheet name="План" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'План'!$A$1:$AK$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'План'!$A$1:$AL$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -603,7 +603,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="A1:G31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -635,7 +635,7 @@
     <row r="4" ht="36" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Все команды заполняют один и тот же Excel. Цвета ячеек больше не означают занятость. Занятость — это даты, числа дней и слово «отпуск».</t>
+          <t>Все команды заполняют один и тот же Excel. Цвета ячеек больше не означают занятость. Занятость — это даты и числа дней. Отпуск отмечается отдельно.</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Тип — деливери / дискавери / ЦКО, либо пусто.</t>
+          <t>Тип — только деливери или дискавери, либо пусто. ЦКО не пишите.</t>
         </is>
       </c>
     </row>
@@ -704,105 +704,112 @@
     <row r="15" ht="36" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Роль — Дизайн / SA / PO / BE / FE / QA / Контент / Отпуск. Если не указать, подставится роль из штата.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
+          <t>Роль — Дизайн / SA / PO / BE / FE / QA / Контент. Если не указать, подставится роль из штата. Отпуск ролью не является.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="36" customHeight="1">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>Отпуск — поставьте «да», если эта строка про нерабочие дни человека. Роль оставьте настоящей (QA, SA, …). Даты начала и окончания — период отпуска.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Начало и Окончание — рабочие даты включительно. Выходные игнорируются.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>Чел-дни — необязательно. Если пусто, считаются все будни между началом и окончанием. Если указано 3 при пяти днях в диапазоне, в план попадут первые 3 будня.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Недели справа — точный вариант, как в таймплане: 1–5 или отпуск. Если заполнены недели, они важнее дат.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="20" customHeight="1">
-      <c r="A19" s="2" t="inlineStr"/>
+          <t>Чел-дни — необязательно и только для работы, не для отпуска. Если пусто, считаются все будни между началом и окончанием. Если указано 3 при пяти днях в диапазоне, в план попадут первые 3 будня.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="36" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Недели справа — занятость работой: 1–5. Если заполнены, они важнее дат. В отпускные недели ничего не ставьте: отпуск уже отмечен колонкой «Отпуск».</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="20" customHeight="1">
-      <c r="A20" s="3" t="inlineStr">
+      <c r="A20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Чего нельзя делать</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="36" customHeight="1">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Не закрашивайте недели цветом вместо числа. Цвет команды в колонке «Команда» ставится сам и в расчёт не идёт.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="36" customHeight="1">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>Не пишите свободным текстом роли (аналитика, фронт, тесты) и не сокращайте имена.</t>
+          <t>Не закрашивайте недели цветом вместо числа. Цвет команды в колонке «Команда» ставится сам и в расчёт не идёт.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="36" customHeight="1">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>Не ставьте одну строку на всю команду. Одна строка = один исполнитель × одна задача.</t>
+          <t>Не пишите свободным текстом роли (аналитика, фронт, тесты) и не сокращайте имена.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="36" customHeight="1">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>Не ставьте одну строку на всю команду. Одна строка = один исполнитель × одна задача.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="36" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
           <t>Потребность без человека — выберите «Потребность SA/FE/BE/QA/дизайн/контент». Это спрос без FTE.</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="2" t="inlineStr"/>
-    </row>
     <row r="26" ht="20" customHeight="1">
-      <c r="A26" s="3" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
         <is>
           <t>Отпуска</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="20" customHeight="1">
-      <c r="A27" s="2" t="inlineStr">
-        <is>
-          <t>Роль = Отпуск, либо в неделе напишите «отпуск». Исполнителя укажите из списка.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="20" customHeight="1">
-      <c r="A28" s="2" t="inlineStr"/>
+    <row r="28" ht="36" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>Отдельная строка на человека: роль из списка, в колонке «Отпуск» — да, даты периода. Эти дни у человека не рабочие и в спрос не идут.</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="20" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+      <c r="A29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
         <is>
           <t>Как отдать файл</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="36" customHeight="1">
-      <c r="A30" s="2" t="inlineStr">
+    <row r="31" ht="36" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>Сохраните как .xlsx и пришлите целиком. Можно один общий файл на все команды или по файлу на команду — структура листа «План» должна совпадать.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="30">
+  <mergeCells count="31">
     <mergeCell ref="A14:G14"/>
     <mergeCell ref="A17:G17"/>
     <mergeCell ref="A8:G8"/>
@@ -815,6 +822,7 @@
     <mergeCell ref="A28:G28"/>
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A31:G31"/>
     <mergeCell ref="A24:G24"/>
     <mergeCell ref="A30:G30"/>
     <mergeCell ref="A15:G15"/>
@@ -844,7 +852,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H41"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -853,6 +861,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -886,6 +895,11 @@
           <t>Команды исполнителя</t>
         </is>
       </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Отпуск</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="5" t="inlineStr">
@@ -918,6 +932,11 @@
           <t>Тарифы</t>
         </is>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -957,11 +976,6 @@
           <t>ДГП</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>ЦКО</t>
-        </is>
-      </c>
       <c r="E4" t="inlineStr">
         <is>
           <t>Настя</t>
@@ -1090,11 +1104,6 @@
       <c r="F9" t="inlineStr">
         <is>
           <t>BE</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>Отпуск</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -1607,7 +1616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AK121"/>
+  <dimension ref="A1:AL121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1616,11 +1625,11 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
     <col width="13" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
     <col width="7" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="7" customWidth="1" min="14" max="14"/>
@@ -1647,6 +1656,7 @@
     <col width="7" customWidth="1" min="35" max="35"/>
     <col width="7" customWidth="1" min="36" max="36"/>
     <col width="7" customWidth="1" min="37" max="37"/>
+    <col width="7" customWidth="1" min="38" max="38"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -1682,155 +1692,160 @@
       </c>
       <c r="G1" s="11" t="inlineStr">
         <is>
+          <t>Отпуск</t>
+        </is>
+      </c>
+      <c r="H1" s="11" t="inlineStr">
+        <is>
           <t>Начало</t>
         </is>
       </c>
-      <c r="H1" s="11" t="inlineStr">
+      <c r="I1" s="11" t="inlineStr">
         <is>
           <t>Окончание</t>
         </is>
       </c>
-      <c r="I1" s="11" t="inlineStr">
+      <c r="J1" s="11" t="inlineStr">
         <is>
           <t>Чел-дни</t>
         </is>
       </c>
-      <c r="J1" s="11" t="inlineStr">
+      <c r="K1" s="11" t="inlineStr">
         <is>
           <t>Примечание</t>
         </is>
       </c>
-      <c r="K1" s="11" t="inlineStr">
+      <c r="L1" s="11" t="inlineStr">
         <is>
           <t>29.06</t>
         </is>
       </c>
-      <c r="L1" s="11" t="inlineStr">
+      <c r="M1" s="11" t="inlineStr">
         <is>
           <t>06.07</t>
         </is>
       </c>
-      <c r="M1" s="11" t="inlineStr">
+      <c r="N1" s="11" t="inlineStr">
         <is>
           <t>13.07</t>
         </is>
       </c>
-      <c r="N1" s="11" t="inlineStr">
+      <c r="O1" s="11" t="inlineStr">
         <is>
           <t>20.07</t>
         </is>
       </c>
-      <c r="O1" s="11" t="inlineStr">
+      <c r="P1" s="11" t="inlineStr">
         <is>
           <t>27.07</t>
         </is>
       </c>
-      <c r="P1" s="11" t="inlineStr">
+      <c r="Q1" s="11" t="inlineStr">
         <is>
           <t>03.08</t>
         </is>
       </c>
-      <c r="Q1" s="11" t="inlineStr">
+      <c r="R1" s="11" t="inlineStr">
         <is>
           <t>10.08</t>
         </is>
       </c>
-      <c r="R1" s="11" t="inlineStr">
+      <c r="S1" s="11" t="inlineStr">
         <is>
           <t>17.08</t>
         </is>
       </c>
-      <c r="S1" s="11" t="inlineStr">
+      <c r="T1" s="11" t="inlineStr">
         <is>
           <t>24.08</t>
         </is>
       </c>
-      <c r="T1" s="11" t="inlineStr">
+      <c r="U1" s="11" t="inlineStr">
         <is>
           <t>31.08</t>
         </is>
       </c>
-      <c r="U1" s="11" t="inlineStr">
+      <c r="V1" s="11" t="inlineStr">
         <is>
           <t>07.09</t>
         </is>
       </c>
-      <c r="V1" s="11" t="inlineStr">
+      <c r="W1" s="11" t="inlineStr">
         <is>
           <t>14.09</t>
         </is>
       </c>
-      <c r="W1" s="11" t="inlineStr">
+      <c r="X1" s="11" t="inlineStr">
         <is>
           <t>21.09</t>
         </is>
       </c>
-      <c r="X1" s="11" t="inlineStr">
+      <c r="Y1" s="11" t="inlineStr">
         <is>
           <t>28.09</t>
         </is>
       </c>
-      <c r="Y1" s="11" t="inlineStr">
+      <c r="Z1" s="11" t="inlineStr">
         <is>
           <t>05.10</t>
         </is>
       </c>
-      <c r="Z1" s="11" t="inlineStr">
+      <c r="AA1" s="11" t="inlineStr">
         <is>
           <t>12.10</t>
         </is>
       </c>
-      <c r="AA1" s="11" t="inlineStr">
+      <c r="AB1" s="11" t="inlineStr">
         <is>
           <t>19.10</t>
         </is>
       </c>
-      <c r="AB1" s="11" t="inlineStr">
+      <c r="AC1" s="11" t="inlineStr">
         <is>
           <t>26.10</t>
         </is>
       </c>
-      <c r="AC1" s="11" t="inlineStr">
+      <c r="AD1" s="11" t="inlineStr">
         <is>
           <t>02.11</t>
         </is>
       </c>
-      <c r="AD1" s="11" t="inlineStr">
+      <c r="AE1" s="11" t="inlineStr">
         <is>
           <t>09.11</t>
         </is>
       </c>
-      <c r="AE1" s="11" t="inlineStr">
+      <c r="AF1" s="11" t="inlineStr">
         <is>
           <t>16.11</t>
         </is>
       </c>
-      <c r="AF1" s="11" t="inlineStr">
+      <c r="AG1" s="11" t="inlineStr">
         <is>
           <t>23.11</t>
         </is>
       </c>
-      <c r="AG1" s="11" t="inlineStr">
+      <c r="AH1" s="11" t="inlineStr">
         <is>
           <t>30.11</t>
         </is>
       </c>
-      <c r="AH1" s="11" t="inlineStr">
+      <c r="AI1" s="11" t="inlineStr">
         <is>
           <t>07.12</t>
         </is>
       </c>
-      <c r="AI1" s="11" t="inlineStr">
+      <c r="AJ1" s="11" t="inlineStr">
         <is>
           <t>14.12</t>
         </is>
       </c>
-      <c r="AJ1" s="11" t="inlineStr">
+      <c r="AK1" s="11" t="inlineStr">
         <is>
           <t>21.12</t>
         </is>
       </c>
-      <c r="AK1" s="11" t="inlineStr">
+      <c r="AL1" s="11" t="inlineStr">
         <is>
           <t>28.12</t>
         </is>
@@ -1863,28 +1878,28 @@
           <t>SA</t>
         </is>
       </c>
-      <c r="G2" s="13" t="n">
+      <c r="G2" s="12" t="inlineStr"/>
+      <c r="H2" s="13" t="n">
         <v>46237</v>
       </c>
-      <c r="H2" s="13" t="n">
+      <c r="I2" s="13" t="n">
         <v>46248</v>
       </c>
-      <c r="I2" s="12" t="n">
+      <c r="J2" s="12" t="n">
         <v>10</v>
       </c>
-      <c r="J2" s="12" t="inlineStr"/>
-      <c r="K2" s="14" t="inlineStr"/>
+      <c r="K2" s="12" t="inlineStr"/>
       <c r="L2" s="14" t="inlineStr"/>
       <c r="M2" s="14" t="inlineStr"/>
       <c r="N2" s="14" t="inlineStr"/>
       <c r="O2" s="14" t="inlineStr"/>
-      <c r="P2" s="14" t="n">
-        <v>5</v>
-      </c>
+      <c r="P2" s="14" t="inlineStr"/>
       <c r="Q2" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="R2" s="14" t="inlineStr"/>
+      <c r="R2" s="14" t="n">
+        <v>5</v>
+      </c>
       <c r="S2" s="14" t="inlineStr"/>
       <c r="T2" s="14" t="inlineStr"/>
       <c r="U2" s="14" t="inlineStr"/>
@@ -1904,6 +1919,7 @@
       <c r="AI2" s="14" t="inlineStr"/>
       <c r="AJ2" s="14" t="inlineStr"/>
       <c r="AK2" s="14" t="inlineStr"/>
+      <c r="AL2" s="14" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -1932,25 +1948,25 @@
           <t>Дизайн</t>
         </is>
       </c>
-      <c r="G3" s="13" t="n">
+      <c r="G3" s="12" t="inlineStr"/>
+      <c r="H3" s="13" t="n">
         <v>46237</v>
       </c>
-      <c r="H3" s="13" t="n">
+      <c r="I3" s="13" t="n">
         <v>46238</v>
       </c>
-      <c r="I3" s="12" t="n">
+      <c r="J3" s="12" t="n">
         <v>2</v>
       </c>
-      <c r="J3" s="12" t="inlineStr"/>
-      <c r="K3" s="14" t="inlineStr"/>
+      <c r="K3" s="12" t="inlineStr"/>
       <c r="L3" s="14" t="inlineStr"/>
       <c r="M3" s="14" t="inlineStr"/>
       <c r="N3" s="14" t="inlineStr"/>
       <c r="O3" s="14" t="inlineStr"/>
-      <c r="P3" s="14" t="n">
+      <c r="P3" s="14" t="inlineStr"/>
+      <c r="Q3" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="Q3" s="14" t="inlineStr"/>
       <c r="R3" s="14" t="inlineStr"/>
       <c r="S3" s="14" t="inlineStr"/>
       <c r="T3" s="14" t="inlineStr"/>
@@ -1971,6 +1987,7 @@
       <c r="AI3" s="14" t="inlineStr"/>
       <c r="AJ3" s="14" t="inlineStr"/>
       <c r="AK3" s="14" t="inlineStr"/>
+      <c r="AL3" s="14" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -1995,28 +2012,28 @@
           <t>Дизайн</t>
         </is>
       </c>
-      <c r="G4" s="13" t="n">
+      <c r="G4" s="12" t="inlineStr"/>
+      <c r="H4" s="13" t="n">
         <v>46237</v>
       </c>
-      <c r="H4" s="13" t="n">
+      <c r="I4" s="13" t="n">
         <v>46248</v>
       </c>
-      <c r="I4" s="12" t="n">
+      <c r="J4" s="12" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="12" t="inlineStr"/>
-      <c r="K4" s="14" t="inlineStr"/>
+      <c r="K4" s="12" t="inlineStr"/>
       <c r="L4" s="14" t="inlineStr"/>
       <c r="M4" s="14" t="inlineStr"/>
       <c r="N4" s="14" t="inlineStr"/>
       <c r="O4" s="14" t="inlineStr"/>
-      <c r="P4" s="14" t="n">
+      <c r="P4" s="14" t="inlineStr"/>
+      <c r="Q4" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="Q4" s="14" t="n">
+      <c r="R4" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="R4" s="14" t="inlineStr"/>
       <c r="S4" s="14" t="inlineStr"/>
       <c r="T4" s="14" t="inlineStr"/>
       <c r="U4" s="14" t="inlineStr"/>
@@ -2036,45 +2053,71 @@
       <c r="AI4" s="14" t="inlineStr"/>
       <c r="AJ4" s="14" t="inlineStr"/>
       <c r="AK4" s="14" t="inlineStr"/>
+      <c r="AL4" s="14" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="15" t="inlineStr"/>
-      <c r="B5" s="15" t="inlineStr"/>
-      <c r="C5" s="15" t="inlineStr"/>
-      <c r="D5" s="15" t="inlineStr"/>
-      <c r="E5" s="15" t="inlineStr"/>
-      <c r="F5" s="15" t="inlineStr"/>
-      <c r="G5" s="16" t="inlineStr"/>
-      <c r="H5" s="16" t="inlineStr"/>
-      <c r="I5" s="15" t="inlineStr"/>
-      <c r="J5" s="15" t="inlineStr"/>
-      <c r="K5" s="17" t="inlineStr"/>
-      <c r="L5" s="17" t="inlineStr"/>
-      <c r="M5" s="17" t="inlineStr"/>
-      <c r="N5" s="17" t="inlineStr"/>
-      <c r="O5" s="17" t="inlineStr"/>
-      <c r="P5" s="17" t="inlineStr"/>
-      <c r="Q5" s="17" t="inlineStr"/>
-      <c r="R5" s="17" t="inlineStr"/>
-      <c r="S5" s="17" t="inlineStr"/>
-      <c r="T5" s="17" t="inlineStr"/>
-      <c r="U5" s="17" t="inlineStr"/>
-      <c r="V5" s="17" t="inlineStr"/>
-      <c r="W5" s="17" t="inlineStr"/>
-      <c r="X5" s="17" t="inlineStr"/>
-      <c r="Y5" s="17" t="inlineStr"/>
-      <c r="Z5" s="17" t="inlineStr"/>
-      <c r="AA5" s="17" t="inlineStr"/>
-      <c r="AB5" s="17" t="inlineStr"/>
-      <c r="AC5" s="17" t="inlineStr"/>
-      <c r="AD5" s="17" t="inlineStr"/>
-      <c r="AE5" s="17" t="inlineStr"/>
-      <c r="AF5" s="17" t="inlineStr"/>
-      <c r="AG5" s="17" t="inlineStr"/>
-      <c r="AH5" s="17" t="inlineStr"/>
-      <c r="AI5" s="17" t="inlineStr"/>
-      <c r="AJ5" s="17" t="inlineStr"/>
-      <c r="AK5" s="17" t="inlineStr"/>
+      <c r="A5" s="12" t="inlineStr">
+        <is>
+          <t>Монетизация</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>ПРИМЕР: отпуск</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr"/>
+      <c r="D5" s="12" t="inlineStr"/>
+      <c r="E5" s="12" t="inlineStr">
+        <is>
+          <t>Роган Татьяна</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="G5" s="12" t="inlineStr">
+        <is>
+          <t>да</t>
+        </is>
+      </c>
+      <c r="H5" s="13" t="n">
+        <v>46272</v>
+      </c>
+      <c r="I5" s="13" t="n">
+        <v>46276</v>
+      </c>
+      <c r="J5" s="12" t="n"/>
+      <c r="K5" s="12" t="inlineStr"/>
+      <c r="L5" s="14" t="inlineStr"/>
+      <c r="M5" s="14" t="inlineStr"/>
+      <c r="N5" s="14" t="inlineStr"/>
+      <c r="O5" s="14" t="inlineStr"/>
+      <c r="P5" s="14" t="inlineStr"/>
+      <c r="Q5" s="14" t="inlineStr"/>
+      <c r="R5" s="14" t="inlineStr"/>
+      <c r="S5" s="14" t="inlineStr"/>
+      <c r="T5" s="14" t="inlineStr"/>
+      <c r="U5" s="14" t="inlineStr"/>
+      <c r="V5" s="14" t="inlineStr"/>
+      <c r="W5" s="14" t="inlineStr"/>
+      <c r="X5" s="14" t="inlineStr"/>
+      <c r="Y5" s="14" t="inlineStr"/>
+      <c r="Z5" s="14" t="inlineStr"/>
+      <c r="AA5" s="14" t="inlineStr"/>
+      <c r="AB5" s="14" t="inlineStr"/>
+      <c r="AC5" s="14" t="inlineStr"/>
+      <c r="AD5" s="14" t="inlineStr"/>
+      <c r="AE5" s="14" t="inlineStr"/>
+      <c r="AF5" s="14" t="inlineStr"/>
+      <c r="AG5" s="14" t="inlineStr"/>
+      <c r="AH5" s="14" t="inlineStr"/>
+      <c r="AI5" s="14" t="inlineStr"/>
+      <c r="AJ5" s="14" t="inlineStr"/>
+      <c r="AK5" s="14" t="inlineStr"/>
+      <c r="AL5" s="14" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr"/>
@@ -2083,11 +2126,11 @@
       <c r="D6" s="15" t="inlineStr"/>
       <c r="E6" s="15" t="inlineStr"/>
       <c r="F6" s="15" t="inlineStr"/>
-      <c r="G6" s="16" t="inlineStr"/>
+      <c r="G6" s="15" t="inlineStr"/>
       <c r="H6" s="16" t="inlineStr"/>
-      <c r="I6" s="15" t="inlineStr"/>
+      <c r="I6" s="16" t="inlineStr"/>
       <c r="J6" s="15" t="inlineStr"/>
-      <c r="K6" s="17" t="inlineStr"/>
+      <c r="K6" s="15" t="inlineStr"/>
       <c r="L6" s="17" t="inlineStr"/>
       <c r="M6" s="17" t="inlineStr"/>
       <c r="N6" s="17" t="inlineStr"/>
@@ -2114,6 +2157,7 @@
       <c r="AI6" s="17" t="inlineStr"/>
       <c r="AJ6" s="17" t="inlineStr"/>
       <c r="AK6" s="17" t="inlineStr"/>
+      <c r="AL6" s="17" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr"/>
@@ -2122,11 +2166,11 @@
       <c r="D7" s="15" t="inlineStr"/>
       <c r="E7" s="15" t="inlineStr"/>
       <c r="F7" s="15" t="inlineStr"/>
-      <c r="G7" s="16" t="inlineStr"/>
+      <c r="G7" s="15" t="inlineStr"/>
       <c r="H7" s="16" t="inlineStr"/>
-      <c r="I7" s="15" t="inlineStr"/>
+      <c r="I7" s="16" t="inlineStr"/>
       <c r="J7" s="15" t="inlineStr"/>
-      <c r="K7" s="17" t="inlineStr"/>
+      <c r="K7" s="15" t="inlineStr"/>
       <c r="L7" s="17" t="inlineStr"/>
       <c r="M7" s="17" t="inlineStr"/>
       <c r="N7" s="17" t="inlineStr"/>
@@ -2153,6 +2197,7 @@
       <c r="AI7" s="17" t="inlineStr"/>
       <c r="AJ7" s="17" t="inlineStr"/>
       <c r="AK7" s="17" t="inlineStr"/>
+      <c r="AL7" s="17" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr"/>
@@ -2161,11 +2206,11 @@
       <c r="D8" s="15" t="inlineStr"/>
       <c r="E8" s="15" t="inlineStr"/>
       <c r="F8" s="15" t="inlineStr"/>
-      <c r="G8" s="16" t="inlineStr"/>
+      <c r="G8" s="15" t="inlineStr"/>
       <c r="H8" s="16" t="inlineStr"/>
-      <c r="I8" s="15" t="inlineStr"/>
+      <c r="I8" s="16" t="inlineStr"/>
       <c r="J8" s="15" t="inlineStr"/>
-      <c r="K8" s="17" t="inlineStr"/>
+      <c r="K8" s="15" t="inlineStr"/>
       <c r="L8" s="17" t="inlineStr"/>
       <c r="M8" s="17" t="inlineStr"/>
       <c r="N8" s="17" t="inlineStr"/>
@@ -2192,6 +2237,7 @@
       <c r="AI8" s="17" t="inlineStr"/>
       <c r="AJ8" s="17" t="inlineStr"/>
       <c r="AK8" s="17" t="inlineStr"/>
+      <c r="AL8" s="17" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr"/>
@@ -2200,11 +2246,11 @@
       <c r="D9" s="15" t="inlineStr"/>
       <c r="E9" s="15" t="inlineStr"/>
       <c r="F9" s="15" t="inlineStr"/>
-      <c r="G9" s="16" t="inlineStr"/>
+      <c r="G9" s="15" t="inlineStr"/>
       <c r="H9" s="16" t="inlineStr"/>
-      <c r="I9" s="15" t="inlineStr"/>
+      <c r="I9" s="16" t="inlineStr"/>
       <c r="J9" s="15" t="inlineStr"/>
-      <c r="K9" s="17" t="inlineStr"/>
+      <c r="K9" s="15" t="inlineStr"/>
       <c r="L9" s="17" t="inlineStr"/>
       <c r="M9" s="17" t="inlineStr"/>
       <c r="N9" s="17" t="inlineStr"/>
@@ -2231,6 +2277,7 @@
       <c r="AI9" s="17" t="inlineStr"/>
       <c r="AJ9" s="17" t="inlineStr"/>
       <c r="AK9" s="17" t="inlineStr"/>
+      <c r="AL9" s="17" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr"/>
@@ -2239,11 +2286,11 @@
       <c r="D10" s="15" t="inlineStr"/>
       <c r="E10" s="15" t="inlineStr"/>
       <c r="F10" s="15" t="inlineStr"/>
-      <c r="G10" s="16" t="inlineStr"/>
+      <c r="G10" s="15" t="inlineStr"/>
       <c r="H10" s="16" t="inlineStr"/>
-      <c r="I10" s="15" t="inlineStr"/>
+      <c r="I10" s="16" t="inlineStr"/>
       <c r="J10" s="15" t="inlineStr"/>
-      <c r="K10" s="17" t="inlineStr"/>
+      <c r="K10" s="15" t="inlineStr"/>
       <c r="L10" s="17" t="inlineStr"/>
       <c r="M10" s="17" t="inlineStr"/>
       <c r="N10" s="17" t="inlineStr"/>
@@ -2270,6 +2317,7 @@
       <c r="AI10" s="17" t="inlineStr"/>
       <c r="AJ10" s="17" t="inlineStr"/>
       <c r="AK10" s="17" t="inlineStr"/>
+      <c r="AL10" s="17" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr"/>
@@ -2278,11 +2326,11 @@
       <c r="D11" s="15" t="inlineStr"/>
       <c r="E11" s="15" t="inlineStr"/>
       <c r="F11" s="15" t="inlineStr"/>
-      <c r="G11" s="16" t="inlineStr"/>
+      <c r="G11" s="15" t="inlineStr"/>
       <c r="H11" s="16" t="inlineStr"/>
-      <c r="I11" s="15" t="inlineStr"/>
+      <c r="I11" s="16" t="inlineStr"/>
       <c r="J11" s="15" t="inlineStr"/>
-      <c r="K11" s="17" t="inlineStr"/>
+      <c r="K11" s="15" t="inlineStr"/>
       <c r="L11" s="17" t="inlineStr"/>
       <c r="M11" s="17" t="inlineStr"/>
       <c r="N11" s="17" t="inlineStr"/>
@@ -2309,6 +2357,7 @@
       <c r="AI11" s="17" t="inlineStr"/>
       <c r="AJ11" s="17" t="inlineStr"/>
       <c r="AK11" s="17" t="inlineStr"/>
+      <c r="AL11" s="17" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr"/>
@@ -2317,11 +2366,11 @@
       <c r="D12" s="15" t="inlineStr"/>
       <c r="E12" s="15" t="inlineStr"/>
       <c r="F12" s="15" t="inlineStr"/>
-      <c r="G12" s="16" t="inlineStr"/>
+      <c r="G12" s="15" t="inlineStr"/>
       <c r="H12" s="16" t="inlineStr"/>
-      <c r="I12" s="15" t="inlineStr"/>
+      <c r="I12" s="16" t="inlineStr"/>
       <c r="J12" s="15" t="inlineStr"/>
-      <c r="K12" s="17" t="inlineStr"/>
+      <c r="K12" s="15" t="inlineStr"/>
       <c r="L12" s="17" t="inlineStr"/>
       <c r="M12" s="17" t="inlineStr"/>
       <c r="N12" s="17" t="inlineStr"/>
@@ -2348,6 +2397,7 @@
       <c r="AI12" s="17" t="inlineStr"/>
       <c r="AJ12" s="17" t="inlineStr"/>
       <c r="AK12" s="17" t="inlineStr"/>
+      <c r="AL12" s="17" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr"/>
@@ -2356,11 +2406,11 @@
       <c r="D13" s="15" t="inlineStr"/>
       <c r="E13" s="15" t="inlineStr"/>
       <c r="F13" s="15" t="inlineStr"/>
-      <c r="G13" s="16" t="inlineStr"/>
+      <c r="G13" s="15" t="inlineStr"/>
       <c r="H13" s="16" t="inlineStr"/>
-      <c r="I13" s="15" t="inlineStr"/>
+      <c r="I13" s="16" t="inlineStr"/>
       <c r="J13" s="15" t="inlineStr"/>
-      <c r="K13" s="17" t="inlineStr"/>
+      <c r="K13" s="15" t="inlineStr"/>
       <c r="L13" s="17" t="inlineStr"/>
       <c r="M13" s="17" t="inlineStr"/>
       <c r="N13" s="17" t="inlineStr"/>
@@ -2387,6 +2437,7 @@
       <c r="AI13" s="17" t="inlineStr"/>
       <c r="AJ13" s="17" t="inlineStr"/>
       <c r="AK13" s="17" t="inlineStr"/>
+      <c r="AL13" s="17" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr"/>
@@ -2395,11 +2446,11 @@
       <c r="D14" s="15" t="inlineStr"/>
       <c r="E14" s="15" t="inlineStr"/>
       <c r="F14" s="15" t="inlineStr"/>
-      <c r="G14" s="16" t="inlineStr"/>
+      <c r="G14" s="15" t="inlineStr"/>
       <c r="H14" s="16" t="inlineStr"/>
-      <c r="I14" s="15" t="inlineStr"/>
+      <c r="I14" s="16" t="inlineStr"/>
       <c r="J14" s="15" t="inlineStr"/>
-      <c r="K14" s="17" t="inlineStr"/>
+      <c r="K14" s="15" t="inlineStr"/>
       <c r="L14" s="17" t="inlineStr"/>
       <c r="M14" s="17" t="inlineStr"/>
       <c r="N14" s="17" t="inlineStr"/>
@@ -2426,6 +2477,7 @@
       <c r="AI14" s="17" t="inlineStr"/>
       <c r="AJ14" s="17" t="inlineStr"/>
       <c r="AK14" s="17" t="inlineStr"/>
+      <c r="AL14" s="17" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr"/>
@@ -2434,11 +2486,11 @@
       <c r="D15" s="15" t="inlineStr"/>
       <c r="E15" s="15" t="inlineStr"/>
       <c r="F15" s="15" t="inlineStr"/>
-      <c r="G15" s="16" t="inlineStr"/>
+      <c r="G15" s="15" t="inlineStr"/>
       <c r="H15" s="16" t="inlineStr"/>
-      <c r="I15" s="15" t="inlineStr"/>
+      <c r="I15" s="16" t="inlineStr"/>
       <c r="J15" s="15" t="inlineStr"/>
-      <c r="K15" s="17" t="inlineStr"/>
+      <c r="K15" s="15" t="inlineStr"/>
       <c r="L15" s="17" t="inlineStr"/>
       <c r="M15" s="17" t="inlineStr"/>
       <c r="N15" s="17" t="inlineStr"/>
@@ -2465,6 +2517,7 @@
       <c r="AI15" s="17" t="inlineStr"/>
       <c r="AJ15" s="17" t="inlineStr"/>
       <c r="AK15" s="17" t="inlineStr"/>
+      <c r="AL15" s="17" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr"/>
@@ -2473,11 +2526,11 @@
       <c r="D16" s="15" t="inlineStr"/>
       <c r="E16" s="15" t="inlineStr"/>
       <c r="F16" s="15" t="inlineStr"/>
-      <c r="G16" s="16" t="inlineStr"/>
+      <c r="G16" s="15" t="inlineStr"/>
       <c r="H16" s="16" t="inlineStr"/>
-      <c r="I16" s="15" t="inlineStr"/>
+      <c r="I16" s="16" t="inlineStr"/>
       <c r="J16" s="15" t="inlineStr"/>
-      <c r="K16" s="17" t="inlineStr"/>
+      <c r="K16" s="15" t="inlineStr"/>
       <c r="L16" s="17" t="inlineStr"/>
       <c r="M16" s="17" t="inlineStr"/>
       <c r="N16" s="17" t="inlineStr"/>
@@ -2504,6 +2557,7 @@
       <c r="AI16" s="17" t="inlineStr"/>
       <c r="AJ16" s="17" t="inlineStr"/>
       <c r="AK16" s="17" t="inlineStr"/>
+      <c r="AL16" s="17" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr"/>
@@ -2512,11 +2566,11 @@
       <c r="D17" s="15" t="inlineStr"/>
       <c r="E17" s="15" t="inlineStr"/>
       <c r="F17" s="15" t="inlineStr"/>
-      <c r="G17" s="16" t="inlineStr"/>
+      <c r="G17" s="15" t="inlineStr"/>
       <c r="H17" s="16" t="inlineStr"/>
-      <c r="I17" s="15" t="inlineStr"/>
+      <c r="I17" s="16" t="inlineStr"/>
       <c r="J17" s="15" t="inlineStr"/>
-      <c r="K17" s="17" t="inlineStr"/>
+      <c r="K17" s="15" t="inlineStr"/>
       <c r="L17" s="17" t="inlineStr"/>
       <c r="M17" s="17" t="inlineStr"/>
       <c r="N17" s="17" t="inlineStr"/>
@@ -2543,6 +2597,7 @@
       <c r="AI17" s="17" t="inlineStr"/>
       <c r="AJ17" s="17" t="inlineStr"/>
       <c r="AK17" s="17" t="inlineStr"/>
+      <c r="AL17" s="17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr"/>
@@ -2551,11 +2606,11 @@
       <c r="D18" s="15" t="inlineStr"/>
       <c r="E18" s="15" t="inlineStr"/>
       <c r="F18" s="15" t="inlineStr"/>
-      <c r="G18" s="16" t="inlineStr"/>
+      <c r="G18" s="15" t="inlineStr"/>
       <c r="H18" s="16" t="inlineStr"/>
-      <c r="I18" s="15" t="inlineStr"/>
+      <c r="I18" s="16" t="inlineStr"/>
       <c r="J18" s="15" t="inlineStr"/>
-      <c r="K18" s="17" t="inlineStr"/>
+      <c r="K18" s="15" t="inlineStr"/>
       <c r="L18" s="17" t="inlineStr"/>
       <c r="M18" s="17" t="inlineStr"/>
       <c r="N18" s="17" t="inlineStr"/>
@@ -2582,6 +2637,7 @@
       <c r="AI18" s="17" t="inlineStr"/>
       <c r="AJ18" s="17" t="inlineStr"/>
       <c r="AK18" s="17" t="inlineStr"/>
+      <c r="AL18" s="17" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr"/>
@@ -2590,11 +2646,11 @@
       <c r="D19" s="15" t="inlineStr"/>
       <c r="E19" s="15" t="inlineStr"/>
       <c r="F19" s="15" t="inlineStr"/>
-      <c r="G19" s="16" t="inlineStr"/>
+      <c r="G19" s="15" t="inlineStr"/>
       <c r="H19" s="16" t="inlineStr"/>
-      <c r="I19" s="15" t="inlineStr"/>
+      <c r="I19" s="16" t="inlineStr"/>
       <c r="J19" s="15" t="inlineStr"/>
-      <c r="K19" s="17" t="inlineStr"/>
+      <c r="K19" s="15" t="inlineStr"/>
       <c r="L19" s="17" t="inlineStr"/>
       <c r="M19" s="17" t="inlineStr"/>
       <c r="N19" s="17" t="inlineStr"/>
@@ -2621,6 +2677,7 @@
       <c r="AI19" s="17" t="inlineStr"/>
       <c r="AJ19" s="17" t="inlineStr"/>
       <c r="AK19" s="17" t="inlineStr"/>
+      <c r="AL19" s="17" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr"/>
@@ -2629,11 +2686,11 @@
       <c r="D20" s="15" t="inlineStr"/>
       <c r="E20" s="15" t="inlineStr"/>
       <c r="F20" s="15" t="inlineStr"/>
-      <c r="G20" s="16" t="inlineStr"/>
+      <c r="G20" s="15" t="inlineStr"/>
       <c r="H20" s="16" t="inlineStr"/>
-      <c r="I20" s="15" t="inlineStr"/>
+      <c r="I20" s="16" t="inlineStr"/>
       <c r="J20" s="15" t="inlineStr"/>
-      <c r="K20" s="17" t="inlineStr"/>
+      <c r="K20" s="15" t="inlineStr"/>
       <c r="L20" s="17" t="inlineStr"/>
       <c r="M20" s="17" t="inlineStr"/>
       <c r="N20" s="17" t="inlineStr"/>
@@ -2660,6 +2717,7 @@
       <c r="AI20" s="17" t="inlineStr"/>
       <c r="AJ20" s="17" t="inlineStr"/>
       <c r="AK20" s="17" t="inlineStr"/>
+      <c r="AL20" s="17" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr"/>
@@ -2668,11 +2726,11 @@
       <c r="D21" s="15" t="inlineStr"/>
       <c r="E21" s="15" t="inlineStr"/>
       <c r="F21" s="15" t="inlineStr"/>
-      <c r="G21" s="16" t="inlineStr"/>
+      <c r="G21" s="15" t="inlineStr"/>
       <c r="H21" s="16" t="inlineStr"/>
-      <c r="I21" s="15" t="inlineStr"/>
+      <c r="I21" s="16" t="inlineStr"/>
       <c r="J21" s="15" t="inlineStr"/>
-      <c r="K21" s="17" t="inlineStr"/>
+      <c r="K21" s="15" t="inlineStr"/>
       <c r="L21" s="17" t="inlineStr"/>
       <c r="M21" s="17" t="inlineStr"/>
       <c r="N21" s="17" t="inlineStr"/>
@@ -2699,6 +2757,7 @@
       <c r="AI21" s="17" t="inlineStr"/>
       <c r="AJ21" s="17" t="inlineStr"/>
       <c r="AK21" s="17" t="inlineStr"/>
+      <c r="AL21" s="17" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr"/>
@@ -2707,11 +2766,11 @@
       <c r="D22" s="15" t="inlineStr"/>
       <c r="E22" s="15" t="inlineStr"/>
       <c r="F22" s="15" t="inlineStr"/>
-      <c r="G22" s="16" t="inlineStr"/>
+      <c r="G22" s="15" t="inlineStr"/>
       <c r="H22" s="16" t="inlineStr"/>
-      <c r="I22" s="15" t="inlineStr"/>
+      <c r="I22" s="16" t="inlineStr"/>
       <c r="J22" s="15" t="inlineStr"/>
-      <c r="K22" s="17" t="inlineStr"/>
+      <c r="K22" s="15" t="inlineStr"/>
       <c r="L22" s="17" t="inlineStr"/>
       <c r="M22" s="17" t="inlineStr"/>
       <c r="N22" s="17" t="inlineStr"/>
@@ -2738,6 +2797,7 @@
       <c r="AI22" s="17" t="inlineStr"/>
       <c r="AJ22" s="17" t="inlineStr"/>
       <c r="AK22" s="17" t="inlineStr"/>
+      <c r="AL22" s="17" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr"/>
@@ -2746,11 +2806,11 @@
       <c r="D23" s="15" t="inlineStr"/>
       <c r="E23" s="15" t="inlineStr"/>
       <c r="F23" s="15" t="inlineStr"/>
-      <c r="G23" s="16" t="inlineStr"/>
+      <c r="G23" s="15" t="inlineStr"/>
       <c r="H23" s="16" t="inlineStr"/>
-      <c r="I23" s="15" t="inlineStr"/>
+      <c r="I23" s="16" t="inlineStr"/>
       <c r="J23" s="15" t="inlineStr"/>
-      <c r="K23" s="17" t="inlineStr"/>
+      <c r="K23" s="15" t="inlineStr"/>
       <c r="L23" s="17" t="inlineStr"/>
       <c r="M23" s="17" t="inlineStr"/>
       <c r="N23" s="17" t="inlineStr"/>
@@ -2777,6 +2837,7 @@
       <c r="AI23" s="17" t="inlineStr"/>
       <c r="AJ23" s="17" t="inlineStr"/>
       <c r="AK23" s="17" t="inlineStr"/>
+      <c r="AL23" s="17" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr"/>
@@ -2785,11 +2846,11 @@
       <c r="D24" s="15" t="inlineStr"/>
       <c r="E24" s="15" t="inlineStr"/>
       <c r="F24" s="15" t="inlineStr"/>
-      <c r="G24" s="16" t="inlineStr"/>
+      <c r="G24" s="15" t="inlineStr"/>
       <c r="H24" s="16" t="inlineStr"/>
-      <c r="I24" s="15" t="inlineStr"/>
+      <c r="I24" s="16" t="inlineStr"/>
       <c r="J24" s="15" t="inlineStr"/>
-      <c r="K24" s="17" t="inlineStr"/>
+      <c r="K24" s="15" t="inlineStr"/>
       <c r="L24" s="17" t="inlineStr"/>
       <c r="M24" s="17" t="inlineStr"/>
       <c r="N24" s="17" t="inlineStr"/>
@@ -2816,6 +2877,7 @@
       <c r="AI24" s="17" t="inlineStr"/>
       <c r="AJ24" s="17" t="inlineStr"/>
       <c r="AK24" s="17" t="inlineStr"/>
+      <c r="AL24" s="17" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr"/>
@@ -2824,11 +2886,11 @@
       <c r="D25" s="15" t="inlineStr"/>
       <c r="E25" s="15" t="inlineStr"/>
       <c r="F25" s="15" t="inlineStr"/>
-      <c r="G25" s="16" t="inlineStr"/>
+      <c r="G25" s="15" t="inlineStr"/>
       <c r="H25" s="16" t="inlineStr"/>
-      <c r="I25" s="15" t="inlineStr"/>
+      <c r="I25" s="16" t="inlineStr"/>
       <c r="J25" s="15" t="inlineStr"/>
-      <c r="K25" s="17" t="inlineStr"/>
+      <c r="K25" s="15" t="inlineStr"/>
       <c r="L25" s="17" t="inlineStr"/>
       <c r="M25" s="17" t="inlineStr"/>
       <c r="N25" s="17" t="inlineStr"/>
@@ -2855,6 +2917,7 @@
       <c r="AI25" s="17" t="inlineStr"/>
       <c r="AJ25" s="17" t="inlineStr"/>
       <c r="AK25" s="17" t="inlineStr"/>
+      <c r="AL25" s="17" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr"/>
@@ -2863,11 +2926,11 @@
       <c r="D26" s="15" t="inlineStr"/>
       <c r="E26" s="15" t="inlineStr"/>
       <c r="F26" s="15" t="inlineStr"/>
-      <c r="G26" s="16" t="inlineStr"/>
+      <c r="G26" s="15" t="inlineStr"/>
       <c r="H26" s="16" t="inlineStr"/>
-      <c r="I26" s="15" t="inlineStr"/>
+      <c r="I26" s="16" t="inlineStr"/>
       <c r="J26" s="15" t="inlineStr"/>
-      <c r="K26" s="17" t="inlineStr"/>
+      <c r="K26" s="15" t="inlineStr"/>
       <c r="L26" s="17" t="inlineStr"/>
       <c r="M26" s="17" t="inlineStr"/>
       <c r="N26" s="17" t="inlineStr"/>
@@ -2894,6 +2957,7 @@
       <c r="AI26" s="17" t="inlineStr"/>
       <c r="AJ26" s="17" t="inlineStr"/>
       <c r="AK26" s="17" t="inlineStr"/>
+      <c r="AL26" s="17" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr"/>
@@ -2902,11 +2966,11 @@
       <c r="D27" s="15" t="inlineStr"/>
       <c r="E27" s="15" t="inlineStr"/>
       <c r="F27" s="15" t="inlineStr"/>
-      <c r="G27" s="16" t="inlineStr"/>
+      <c r="G27" s="15" t="inlineStr"/>
       <c r="H27" s="16" t="inlineStr"/>
-      <c r="I27" s="15" t="inlineStr"/>
+      <c r="I27" s="16" t="inlineStr"/>
       <c r="J27" s="15" t="inlineStr"/>
-      <c r="K27" s="17" t="inlineStr"/>
+      <c r="K27" s="15" t="inlineStr"/>
       <c r="L27" s="17" t="inlineStr"/>
       <c r="M27" s="17" t="inlineStr"/>
       <c r="N27" s="17" t="inlineStr"/>
@@ -2933,6 +2997,7 @@
       <c r="AI27" s="17" t="inlineStr"/>
       <c r="AJ27" s="17" t="inlineStr"/>
       <c r="AK27" s="17" t="inlineStr"/>
+      <c r="AL27" s="17" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr"/>
@@ -2941,11 +3006,11 @@
       <c r="D28" s="15" t="inlineStr"/>
       <c r="E28" s="15" t="inlineStr"/>
       <c r="F28" s="15" t="inlineStr"/>
-      <c r="G28" s="16" t="inlineStr"/>
+      <c r="G28" s="15" t="inlineStr"/>
       <c r="H28" s="16" t="inlineStr"/>
-      <c r="I28" s="15" t="inlineStr"/>
+      <c r="I28" s="16" t="inlineStr"/>
       <c r="J28" s="15" t="inlineStr"/>
-      <c r="K28" s="17" t="inlineStr"/>
+      <c r="K28" s="15" t="inlineStr"/>
       <c r="L28" s="17" t="inlineStr"/>
       <c r="M28" s="17" t="inlineStr"/>
       <c r="N28" s="17" t="inlineStr"/>
@@ -2972,6 +3037,7 @@
       <c r="AI28" s="17" t="inlineStr"/>
       <c r="AJ28" s="17" t="inlineStr"/>
       <c r="AK28" s="17" t="inlineStr"/>
+      <c r="AL28" s="17" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr"/>
@@ -2980,11 +3046,11 @@
       <c r="D29" s="15" t="inlineStr"/>
       <c r="E29" s="15" t="inlineStr"/>
       <c r="F29" s="15" t="inlineStr"/>
-      <c r="G29" s="16" t="inlineStr"/>
+      <c r="G29" s="15" t="inlineStr"/>
       <c r="H29" s="16" t="inlineStr"/>
-      <c r="I29" s="15" t="inlineStr"/>
+      <c r="I29" s="16" t="inlineStr"/>
       <c r="J29" s="15" t="inlineStr"/>
-      <c r="K29" s="17" t="inlineStr"/>
+      <c r="K29" s="15" t="inlineStr"/>
       <c r="L29" s="17" t="inlineStr"/>
       <c r="M29" s="17" t="inlineStr"/>
       <c r="N29" s="17" t="inlineStr"/>
@@ -3011,6 +3077,7 @@
       <c r="AI29" s="17" t="inlineStr"/>
       <c r="AJ29" s="17" t="inlineStr"/>
       <c r="AK29" s="17" t="inlineStr"/>
+      <c r="AL29" s="17" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr"/>
@@ -3019,11 +3086,11 @@
       <c r="D30" s="15" t="inlineStr"/>
       <c r="E30" s="15" t="inlineStr"/>
       <c r="F30" s="15" t="inlineStr"/>
-      <c r="G30" s="16" t="inlineStr"/>
+      <c r="G30" s="15" t="inlineStr"/>
       <c r="H30" s="16" t="inlineStr"/>
-      <c r="I30" s="15" t="inlineStr"/>
+      <c r="I30" s="16" t="inlineStr"/>
       <c r="J30" s="15" t="inlineStr"/>
-      <c r="K30" s="17" t="inlineStr"/>
+      <c r="K30" s="15" t="inlineStr"/>
       <c r="L30" s="17" t="inlineStr"/>
       <c r="M30" s="17" t="inlineStr"/>
       <c r="N30" s="17" t="inlineStr"/>
@@ -3050,6 +3117,7 @@
       <c r="AI30" s="17" t="inlineStr"/>
       <c r="AJ30" s="17" t="inlineStr"/>
       <c r="AK30" s="17" t="inlineStr"/>
+      <c r="AL30" s="17" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr"/>
@@ -3058,11 +3126,11 @@
       <c r="D31" s="15" t="inlineStr"/>
       <c r="E31" s="15" t="inlineStr"/>
       <c r="F31" s="15" t="inlineStr"/>
-      <c r="G31" s="16" t="inlineStr"/>
+      <c r="G31" s="15" t="inlineStr"/>
       <c r="H31" s="16" t="inlineStr"/>
-      <c r="I31" s="15" t="inlineStr"/>
+      <c r="I31" s="16" t="inlineStr"/>
       <c r="J31" s="15" t="inlineStr"/>
-      <c r="K31" s="17" t="inlineStr"/>
+      <c r="K31" s="15" t="inlineStr"/>
       <c r="L31" s="17" t="inlineStr"/>
       <c r="M31" s="17" t="inlineStr"/>
       <c r="N31" s="17" t="inlineStr"/>
@@ -3089,6 +3157,7 @@
       <c r="AI31" s="17" t="inlineStr"/>
       <c r="AJ31" s="17" t="inlineStr"/>
       <c r="AK31" s="17" t="inlineStr"/>
+      <c r="AL31" s="17" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr"/>
@@ -3097,11 +3166,11 @@
       <c r="D32" s="15" t="inlineStr"/>
       <c r="E32" s="15" t="inlineStr"/>
       <c r="F32" s="15" t="inlineStr"/>
-      <c r="G32" s="16" t="inlineStr"/>
+      <c r="G32" s="15" t="inlineStr"/>
       <c r="H32" s="16" t="inlineStr"/>
-      <c r="I32" s="15" t="inlineStr"/>
+      <c r="I32" s="16" t="inlineStr"/>
       <c r="J32" s="15" t="inlineStr"/>
-      <c r="K32" s="17" t="inlineStr"/>
+      <c r="K32" s="15" t="inlineStr"/>
       <c r="L32" s="17" t="inlineStr"/>
       <c r="M32" s="17" t="inlineStr"/>
       <c r="N32" s="17" t="inlineStr"/>
@@ -3128,6 +3197,7 @@
       <c r="AI32" s="17" t="inlineStr"/>
       <c r="AJ32" s="17" t="inlineStr"/>
       <c r="AK32" s="17" t="inlineStr"/>
+      <c r="AL32" s="17" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr"/>
@@ -3136,11 +3206,11 @@
       <c r="D33" s="15" t="inlineStr"/>
       <c r="E33" s="15" t="inlineStr"/>
       <c r="F33" s="15" t="inlineStr"/>
-      <c r="G33" s="16" t="inlineStr"/>
+      <c r="G33" s="15" t="inlineStr"/>
       <c r="H33" s="16" t="inlineStr"/>
-      <c r="I33" s="15" t="inlineStr"/>
+      <c r="I33" s="16" t="inlineStr"/>
       <c r="J33" s="15" t="inlineStr"/>
-      <c r="K33" s="17" t="inlineStr"/>
+      <c r="K33" s="15" t="inlineStr"/>
       <c r="L33" s="17" t="inlineStr"/>
       <c r="M33" s="17" t="inlineStr"/>
       <c r="N33" s="17" t="inlineStr"/>
@@ -3167,6 +3237,7 @@
       <c r="AI33" s="17" t="inlineStr"/>
       <c r="AJ33" s="17" t="inlineStr"/>
       <c r="AK33" s="17" t="inlineStr"/>
+      <c r="AL33" s="17" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr"/>
@@ -3175,11 +3246,11 @@
       <c r="D34" s="15" t="inlineStr"/>
       <c r="E34" s="15" t="inlineStr"/>
       <c r="F34" s="15" t="inlineStr"/>
-      <c r="G34" s="16" t="inlineStr"/>
+      <c r="G34" s="15" t="inlineStr"/>
       <c r="H34" s="16" t="inlineStr"/>
-      <c r="I34" s="15" t="inlineStr"/>
+      <c r="I34" s="16" t="inlineStr"/>
       <c r="J34" s="15" t="inlineStr"/>
-      <c r="K34" s="17" t="inlineStr"/>
+      <c r="K34" s="15" t="inlineStr"/>
       <c r="L34" s="17" t="inlineStr"/>
       <c r="M34" s="17" t="inlineStr"/>
       <c r="N34" s="17" t="inlineStr"/>
@@ -3206,6 +3277,7 @@
       <c r="AI34" s="17" t="inlineStr"/>
       <c r="AJ34" s="17" t="inlineStr"/>
       <c r="AK34" s="17" t="inlineStr"/>
+      <c r="AL34" s="17" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr"/>
@@ -3214,11 +3286,11 @@
       <c r="D35" s="15" t="inlineStr"/>
       <c r="E35" s="15" t="inlineStr"/>
       <c r="F35" s="15" t="inlineStr"/>
-      <c r="G35" s="16" t="inlineStr"/>
+      <c r="G35" s="15" t="inlineStr"/>
       <c r="H35" s="16" t="inlineStr"/>
-      <c r="I35" s="15" t="inlineStr"/>
+      <c r="I35" s="16" t="inlineStr"/>
       <c r="J35" s="15" t="inlineStr"/>
-      <c r="K35" s="17" t="inlineStr"/>
+      <c r="K35" s="15" t="inlineStr"/>
       <c r="L35" s="17" t="inlineStr"/>
       <c r="M35" s="17" t="inlineStr"/>
       <c r="N35" s="17" t="inlineStr"/>
@@ -3245,6 +3317,7 @@
       <c r="AI35" s="17" t="inlineStr"/>
       <c r="AJ35" s="17" t="inlineStr"/>
       <c r="AK35" s="17" t="inlineStr"/>
+      <c r="AL35" s="17" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="15" t="inlineStr"/>
@@ -3253,11 +3326,11 @@
       <c r="D36" s="15" t="inlineStr"/>
       <c r="E36" s="15" t="inlineStr"/>
       <c r="F36" s="15" t="inlineStr"/>
-      <c r="G36" s="16" t="inlineStr"/>
+      <c r="G36" s="15" t="inlineStr"/>
       <c r="H36" s="16" t="inlineStr"/>
-      <c r="I36" s="15" t="inlineStr"/>
+      <c r="I36" s="16" t="inlineStr"/>
       <c r="J36" s="15" t="inlineStr"/>
-      <c r="K36" s="17" t="inlineStr"/>
+      <c r="K36" s="15" t="inlineStr"/>
       <c r="L36" s="17" t="inlineStr"/>
       <c r="M36" s="17" t="inlineStr"/>
       <c r="N36" s="17" t="inlineStr"/>
@@ -3284,6 +3357,7 @@
       <c r="AI36" s="17" t="inlineStr"/>
       <c r="AJ36" s="17" t="inlineStr"/>
       <c r="AK36" s="17" t="inlineStr"/>
+      <c r="AL36" s="17" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="15" t="inlineStr"/>
@@ -3292,11 +3366,11 @@
       <c r="D37" s="15" t="inlineStr"/>
       <c r="E37" s="15" t="inlineStr"/>
       <c r="F37" s="15" t="inlineStr"/>
-      <c r="G37" s="16" t="inlineStr"/>
+      <c r="G37" s="15" t="inlineStr"/>
       <c r="H37" s="16" t="inlineStr"/>
-      <c r="I37" s="15" t="inlineStr"/>
+      <c r="I37" s="16" t="inlineStr"/>
       <c r="J37" s="15" t="inlineStr"/>
-      <c r="K37" s="17" t="inlineStr"/>
+      <c r="K37" s="15" t="inlineStr"/>
       <c r="L37" s="17" t="inlineStr"/>
       <c r="M37" s="17" t="inlineStr"/>
       <c r="N37" s="17" t="inlineStr"/>
@@ -3323,6 +3397,7 @@
       <c r="AI37" s="17" t="inlineStr"/>
       <c r="AJ37" s="17" t="inlineStr"/>
       <c r="AK37" s="17" t="inlineStr"/>
+      <c r="AL37" s="17" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="15" t="inlineStr"/>
@@ -3331,11 +3406,11 @@
       <c r="D38" s="15" t="inlineStr"/>
       <c r="E38" s="15" t="inlineStr"/>
       <c r="F38" s="15" t="inlineStr"/>
-      <c r="G38" s="16" t="inlineStr"/>
+      <c r="G38" s="15" t="inlineStr"/>
       <c r="H38" s="16" t="inlineStr"/>
-      <c r="I38" s="15" t="inlineStr"/>
+      <c r="I38" s="16" t="inlineStr"/>
       <c r="J38" s="15" t="inlineStr"/>
-      <c r="K38" s="17" t="inlineStr"/>
+      <c r="K38" s="15" t="inlineStr"/>
       <c r="L38" s="17" t="inlineStr"/>
       <c r="M38" s="17" t="inlineStr"/>
       <c r="N38" s="17" t="inlineStr"/>
@@ -3362,6 +3437,7 @@
       <c r="AI38" s="17" t="inlineStr"/>
       <c r="AJ38" s="17" t="inlineStr"/>
       <c r="AK38" s="17" t="inlineStr"/>
+      <c r="AL38" s="17" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr"/>
@@ -3370,11 +3446,11 @@
       <c r="D39" s="15" t="inlineStr"/>
       <c r="E39" s="15" t="inlineStr"/>
       <c r="F39" s="15" t="inlineStr"/>
-      <c r="G39" s="16" t="inlineStr"/>
+      <c r="G39" s="15" t="inlineStr"/>
       <c r="H39" s="16" t="inlineStr"/>
-      <c r="I39" s="15" t="inlineStr"/>
+      <c r="I39" s="16" t="inlineStr"/>
       <c r="J39" s="15" t="inlineStr"/>
-      <c r="K39" s="17" t="inlineStr"/>
+      <c r="K39" s="15" t="inlineStr"/>
       <c r="L39" s="17" t="inlineStr"/>
       <c r="M39" s="17" t="inlineStr"/>
       <c r="N39" s="17" t="inlineStr"/>
@@ -3401,6 +3477,7 @@
       <c r="AI39" s="17" t="inlineStr"/>
       <c r="AJ39" s="17" t="inlineStr"/>
       <c r="AK39" s="17" t="inlineStr"/>
+      <c r="AL39" s="17" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="15" t="inlineStr"/>
@@ -3409,11 +3486,11 @@
       <c r="D40" s="15" t="inlineStr"/>
       <c r="E40" s="15" t="inlineStr"/>
       <c r="F40" s="15" t="inlineStr"/>
-      <c r="G40" s="16" t="inlineStr"/>
+      <c r="G40" s="15" t="inlineStr"/>
       <c r="H40" s="16" t="inlineStr"/>
-      <c r="I40" s="15" t="inlineStr"/>
+      <c r="I40" s="16" t="inlineStr"/>
       <c r="J40" s="15" t="inlineStr"/>
-      <c r="K40" s="17" t="inlineStr"/>
+      <c r="K40" s="15" t="inlineStr"/>
       <c r="L40" s="17" t="inlineStr"/>
       <c r="M40" s="17" t="inlineStr"/>
       <c r="N40" s="17" t="inlineStr"/>
@@ -3440,6 +3517,7 @@
       <c r="AI40" s="17" t="inlineStr"/>
       <c r="AJ40" s="17" t="inlineStr"/>
       <c r="AK40" s="17" t="inlineStr"/>
+      <c r="AL40" s="17" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="15" t="inlineStr"/>
@@ -3448,11 +3526,11 @@
       <c r="D41" s="15" t="inlineStr"/>
       <c r="E41" s="15" t="inlineStr"/>
       <c r="F41" s="15" t="inlineStr"/>
-      <c r="G41" s="16" t="inlineStr"/>
+      <c r="G41" s="15" t="inlineStr"/>
       <c r="H41" s="16" t="inlineStr"/>
-      <c r="I41" s="15" t="inlineStr"/>
+      <c r="I41" s="16" t="inlineStr"/>
       <c r="J41" s="15" t="inlineStr"/>
-      <c r="K41" s="17" t="inlineStr"/>
+      <c r="K41" s="15" t="inlineStr"/>
       <c r="L41" s="17" t="inlineStr"/>
       <c r="M41" s="17" t="inlineStr"/>
       <c r="N41" s="17" t="inlineStr"/>
@@ -3479,6 +3557,7 @@
       <c r="AI41" s="17" t="inlineStr"/>
       <c r="AJ41" s="17" t="inlineStr"/>
       <c r="AK41" s="17" t="inlineStr"/>
+      <c r="AL41" s="17" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="15" t="inlineStr"/>
@@ -3487,11 +3566,11 @@
       <c r="D42" s="15" t="inlineStr"/>
       <c r="E42" s="15" t="inlineStr"/>
       <c r="F42" s="15" t="inlineStr"/>
-      <c r="G42" s="16" t="inlineStr"/>
+      <c r="G42" s="15" t="inlineStr"/>
       <c r="H42" s="16" t="inlineStr"/>
-      <c r="I42" s="15" t="inlineStr"/>
+      <c r="I42" s="16" t="inlineStr"/>
       <c r="J42" s="15" t="inlineStr"/>
-      <c r="K42" s="17" t="inlineStr"/>
+      <c r="K42" s="15" t="inlineStr"/>
       <c r="L42" s="17" t="inlineStr"/>
       <c r="M42" s="17" t="inlineStr"/>
       <c r="N42" s="17" t="inlineStr"/>
@@ -3518,6 +3597,7 @@
       <c r="AI42" s="17" t="inlineStr"/>
       <c r="AJ42" s="17" t="inlineStr"/>
       <c r="AK42" s="17" t="inlineStr"/>
+      <c r="AL42" s="17" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="15" t="inlineStr"/>
@@ -3526,11 +3606,11 @@
       <c r="D43" s="15" t="inlineStr"/>
       <c r="E43" s="15" t="inlineStr"/>
       <c r="F43" s="15" t="inlineStr"/>
-      <c r="G43" s="16" t="inlineStr"/>
+      <c r="G43" s="15" t="inlineStr"/>
       <c r="H43" s="16" t="inlineStr"/>
-      <c r="I43" s="15" t="inlineStr"/>
+      <c r="I43" s="16" t="inlineStr"/>
       <c r="J43" s="15" t="inlineStr"/>
-      <c r="K43" s="17" t="inlineStr"/>
+      <c r="K43" s="15" t="inlineStr"/>
       <c r="L43" s="17" t="inlineStr"/>
       <c r="M43" s="17" t="inlineStr"/>
       <c r="N43" s="17" t="inlineStr"/>
@@ -3557,6 +3637,7 @@
       <c r="AI43" s="17" t="inlineStr"/>
       <c r="AJ43" s="17" t="inlineStr"/>
       <c r="AK43" s="17" t="inlineStr"/>
+      <c r="AL43" s="17" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="15" t="inlineStr"/>
@@ -3565,11 +3646,11 @@
       <c r="D44" s="15" t="inlineStr"/>
       <c r="E44" s="15" t="inlineStr"/>
       <c r="F44" s="15" t="inlineStr"/>
-      <c r="G44" s="16" t="inlineStr"/>
+      <c r="G44" s="15" t="inlineStr"/>
       <c r="H44" s="16" t="inlineStr"/>
-      <c r="I44" s="15" t="inlineStr"/>
+      <c r="I44" s="16" t="inlineStr"/>
       <c r="J44" s="15" t="inlineStr"/>
-      <c r="K44" s="17" t="inlineStr"/>
+      <c r="K44" s="15" t="inlineStr"/>
       <c r="L44" s="17" t="inlineStr"/>
       <c r="M44" s="17" t="inlineStr"/>
       <c r="N44" s="17" t="inlineStr"/>
@@ -3596,6 +3677,7 @@
       <c r="AI44" s="17" t="inlineStr"/>
       <c r="AJ44" s="17" t="inlineStr"/>
       <c r="AK44" s="17" t="inlineStr"/>
+      <c r="AL44" s="17" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="15" t="inlineStr"/>
@@ -3604,11 +3686,11 @@
       <c r="D45" s="15" t="inlineStr"/>
       <c r="E45" s="15" t="inlineStr"/>
       <c r="F45" s="15" t="inlineStr"/>
-      <c r="G45" s="16" t="inlineStr"/>
+      <c r="G45" s="15" t="inlineStr"/>
       <c r="H45" s="16" t="inlineStr"/>
-      <c r="I45" s="15" t="inlineStr"/>
+      <c r="I45" s="16" t="inlineStr"/>
       <c r="J45" s="15" t="inlineStr"/>
-      <c r="K45" s="17" t="inlineStr"/>
+      <c r="K45" s="15" t="inlineStr"/>
       <c r="L45" s="17" t="inlineStr"/>
       <c r="M45" s="17" t="inlineStr"/>
       <c r="N45" s="17" t="inlineStr"/>
@@ -3635,6 +3717,7 @@
       <c r="AI45" s="17" t="inlineStr"/>
       <c r="AJ45" s="17" t="inlineStr"/>
       <c r="AK45" s="17" t="inlineStr"/>
+      <c r="AL45" s="17" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="15" t="inlineStr"/>
@@ -3643,11 +3726,11 @@
       <c r="D46" s="15" t="inlineStr"/>
       <c r="E46" s="15" t="inlineStr"/>
       <c r="F46" s="15" t="inlineStr"/>
-      <c r="G46" s="16" t="inlineStr"/>
+      <c r="G46" s="15" t="inlineStr"/>
       <c r="H46" s="16" t="inlineStr"/>
-      <c r="I46" s="15" t="inlineStr"/>
+      <c r="I46" s="16" t="inlineStr"/>
       <c r="J46" s="15" t="inlineStr"/>
-      <c r="K46" s="17" t="inlineStr"/>
+      <c r="K46" s="15" t="inlineStr"/>
       <c r="L46" s="17" t="inlineStr"/>
       <c r="M46" s="17" t="inlineStr"/>
       <c r="N46" s="17" t="inlineStr"/>
@@ -3674,6 +3757,7 @@
       <c r="AI46" s="17" t="inlineStr"/>
       <c r="AJ46" s="17" t="inlineStr"/>
       <c r="AK46" s="17" t="inlineStr"/>
+      <c r="AL46" s="17" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="15" t="inlineStr"/>
@@ -3682,11 +3766,11 @@
       <c r="D47" s="15" t="inlineStr"/>
       <c r="E47" s="15" t="inlineStr"/>
       <c r="F47" s="15" t="inlineStr"/>
-      <c r="G47" s="16" t="inlineStr"/>
+      <c r="G47" s="15" t="inlineStr"/>
       <c r="H47" s="16" t="inlineStr"/>
-      <c r="I47" s="15" t="inlineStr"/>
+      <c r="I47" s="16" t="inlineStr"/>
       <c r="J47" s="15" t="inlineStr"/>
-      <c r="K47" s="17" t="inlineStr"/>
+      <c r="K47" s="15" t="inlineStr"/>
       <c r="L47" s="17" t="inlineStr"/>
       <c r="M47" s="17" t="inlineStr"/>
       <c r="N47" s="17" t="inlineStr"/>
@@ -3713,6 +3797,7 @@
       <c r="AI47" s="17" t="inlineStr"/>
       <c r="AJ47" s="17" t="inlineStr"/>
       <c r="AK47" s="17" t="inlineStr"/>
+      <c r="AL47" s="17" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" s="15" t="inlineStr"/>
@@ -3721,11 +3806,11 @@
       <c r="D48" s="15" t="inlineStr"/>
       <c r="E48" s="15" t="inlineStr"/>
       <c r="F48" s="15" t="inlineStr"/>
-      <c r="G48" s="16" t="inlineStr"/>
+      <c r="G48" s="15" t="inlineStr"/>
       <c r="H48" s="16" t="inlineStr"/>
-      <c r="I48" s="15" t="inlineStr"/>
+      <c r="I48" s="16" t="inlineStr"/>
       <c r="J48" s="15" t="inlineStr"/>
-      <c r="K48" s="17" t="inlineStr"/>
+      <c r="K48" s="15" t="inlineStr"/>
       <c r="L48" s="17" t="inlineStr"/>
       <c r="M48" s="17" t="inlineStr"/>
       <c r="N48" s="17" t="inlineStr"/>
@@ -3752,6 +3837,7 @@
       <c r="AI48" s="17" t="inlineStr"/>
       <c r="AJ48" s="17" t="inlineStr"/>
       <c r="AK48" s="17" t="inlineStr"/>
+      <c r="AL48" s="17" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" s="15" t="inlineStr"/>
@@ -3760,11 +3846,11 @@
       <c r="D49" s="15" t="inlineStr"/>
       <c r="E49" s="15" t="inlineStr"/>
       <c r="F49" s="15" t="inlineStr"/>
-      <c r="G49" s="16" t="inlineStr"/>
+      <c r="G49" s="15" t="inlineStr"/>
       <c r="H49" s="16" t="inlineStr"/>
-      <c r="I49" s="15" t="inlineStr"/>
+      <c r="I49" s="16" t="inlineStr"/>
       <c r="J49" s="15" t="inlineStr"/>
-      <c r="K49" s="17" t="inlineStr"/>
+      <c r="K49" s="15" t="inlineStr"/>
       <c r="L49" s="17" t="inlineStr"/>
       <c r="M49" s="17" t="inlineStr"/>
       <c r="N49" s="17" t="inlineStr"/>
@@ -3791,6 +3877,7 @@
       <c r="AI49" s="17" t="inlineStr"/>
       <c r="AJ49" s="17" t="inlineStr"/>
       <c r="AK49" s="17" t="inlineStr"/>
+      <c r="AL49" s="17" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" s="15" t="inlineStr"/>
@@ -3799,11 +3886,11 @@
       <c r="D50" s="15" t="inlineStr"/>
       <c r="E50" s="15" t="inlineStr"/>
       <c r="F50" s="15" t="inlineStr"/>
-      <c r="G50" s="16" t="inlineStr"/>
+      <c r="G50" s="15" t="inlineStr"/>
       <c r="H50" s="16" t="inlineStr"/>
-      <c r="I50" s="15" t="inlineStr"/>
+      <c r="I50" s="16" t="inlineStr"/>
       <c r="J50" s="15" t="inlineStr"/>
-      <c r="K50" s="17" t="inlineStr"/>
+      <c r="K50" s="15" t="inlineStr"/>
       <c r="L50" s="17" t="inlineStr"/>
       <c r="M50" s="17" t="inlineStr"/>
       <c r="N50" s="17" t="inlineStr"/>
@@ -3830,6 +3917,7 @@
       <c r="AI50" s="17" t="inlineStr"/>
       <c r="AJ50" s="17" t="inlineStr"/>
       <c r="AK50" s="17" t="inlineStr"/>
+      <c r="AL50" s="17" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" s="15" t="inlineStr"/>
@@ -3838,11 +3926,11 @@
       <c r="D51" s="15" t="inlineStr"/>
       <c r="E51" s="15" t="inlineStr"/>
       <c r="F51" s="15" t="inlineStr"/>
-      <c r="G51" s="16" t="inlineStr"/>
+      <c r="G51" s="15" t="inlineStr"/>
       <c r="H51" s="16" t="inlineStr"/>
-      <c r="I51" s="15" t="inlineStr"/>
+      <c r="I51" s="16" t="inlineStr"/>
       <c r="J51" s="15" t="inlineStr"/>
-      <c r="K51" s="17" t="inlineStr"/>
+      <c r="K51" s="15" t="inlineStr"/>
       <c r="L51" s="17" t="inlineStr"/>
       <c r="M51" s="17" t="inlineStr"/>
       <c r="N51" s="17" t="inlineStr"/>
@@ -3869,6 +3957,7 @@
       <c r="AI51" s="17" t="inlineStr"/>
       <c r="AJ51" s="17" t="inlineStr"/>
       <c r="AK51" s="17" t="inlineStr"/>
+      <c r="AL51" s="17" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" s="15" t="inlineStr"/>
@@ -3877,11 +3966,11 @@
       <c r="D52" s="15" t="inlineStr"/>
       <c r="E52" s="15" t="inlineStr"/>
       <c r="F52" s="15" t="inlineStr"/>
-      <c r="G52" s="16" t="inlineStr"/>
+      <c r="G52" s="15" t="inlineStr"/>
       <c r="H52" s="16" t="inlineStr"/>
-      <c r="I52" s="15" t="inlineStr"/>
+      <c r="I52" s="16" t="inlineStr"/>
       <c r="J52" s="15" t="inlineStr"/>
-      <c r="K52" s="17" t="inlineStr"/>
+      <c r="K52" s="15" t="inlineStr"/>
       <c r="L52" s="17" t="inlineStr"/>
       <c r="M52" s="17" t="inlineStr"/>
       <c r="N52" s="17" t="inlineStr"/>
@@ -3908,6 +3997,7 @@
       <c r="AI52" s="17" t="inlineStr"/>
       <c r="AJ52" s="17" t="inlineStr"/>
       <c r="AK52" s="17" t="inlineStr"/>
+      <c r="AL52" s="17" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" s="15" t="inlineStr"/>
@@ -3916,11 +4006,11 @@
       <c r="D53" s="15" t="inlineStr"/>
       <c r="E53" s="15" t="inlineStr"/>
       <c r="F53" s="15" t="inlineStr"/>
-      <c r="G53" s="16" t="inlineStr"/>
+      <c r="G53" s="15" t="inlineStr"/>
       <c r="H53" s="16" t="inlineStr"/>
-      <c r="I53" s="15" t="inlineStr"/>
+      <c r="I53" s="16" t="inlineStr"/>
       <c r="J53" s="15" t="inlineStr"/>
-      <c r="K53" s="17" t="inlineStr"/>
+      <c r="K53" s="15" t="inlineStr"/>
       <c r="L53" s="17" t="inlineStr"/>
       <c r="M53" s="17" t="inlineStr"/>
       <c r="N53" s="17" t="inlineStr"/>
@@ -3947,6 +4037,7 @@
       <c r="AI53" s="17" t="inlineStr"/>
       <c r="AJ53" s="17" t="inlineStr"/>
       <c r="AK53" s="17" t="inlineStr"/>
+      <c r="AL53" s="17" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" s="15" t="inlineStr"/>
@@ -3955,11 +4046,11 @@
       <c r="D54" s="15" t="inlineStr"/>
       <c r="E54" s="15" t="inlineStr"/>
       <c r="F54" s="15" t="inlineStr"/>
-      <c r="G54" s="16" t="inlineStr"/>
+      <c r="G54" s="15" t="inlineStr"/>
       <c r="H54" s="16" t="inlineStr"/>
-      <c r="I54" s="15" t="inlineStr"/>
+      <c r="I54" s="16" t="inlineStr"/>
       <c r="J54" s="15" t="inlineStr"/>
-      <c r="K54" s="17" t="inlineStr"/>
+      <c r="K54" s="15" t="inlineStr"/>
       <c r="L54" s="17" t="inlineStr"/>
       <c r="M54" s="17" t="inlineStr"/>
       <c r="N54" s="17" t="inlineStr"/>
@@ -3986,6 +4077,7 @@
       <c r="AI54" s="17" t="inlineStr"/>
       <c r="AJ54" s="17" t="inlineStr"/>
       <c r="AK54" s="17" t="inlineStr"/>
+      <c r="AL54" s="17" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" s="15" t="inlineStr"/>
@@ -3994,11 +4086,11 @@
       <c r="D55" s="15" t="inlineStr"/>
       <c r="E55" s="15" t="inlineStr"/>
       <c r="F55" s="15" t="inlineStr"/>
-      <c r="G55" s="16" t="inlineStr"/>
+      <c r="G55" s="15" t="inlineStr"/>
       <c r="H55" s="16" t="inlineStr"/>
-      <c r="I55" s="15" t="inlineStr"/>
+      <c r="I55" s="16" t="inlineStr"/>
       <c r="J55" s="15" t="inlineStr"/>
-      <c r="K55" s="17" t="inlineStr"/>
+      <c r="K55" s="15" t="inlineStr"/>
       <c r="L55" s="17" t="inlineStr"/>
       <c r="M55" s="17" t="inlineStr"/>
       <c r="N55" s="17" t="inlineStr"/>
@@ -4025,6 +4117,7 @@
       <c r="AI55" s="17" t="inlineStr"/>
       <c r="AJ55" s="17" t="inlineStr"/>
       <c r="AK55" s="17" t="inlineStr"/>
+      <c r="AL55" s="17" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" s="15" t="inlineStr"/>
@@ -4033,11 +4126,11 @@
       <c r="D56" s="15" t="inlineStr"/>
       <c r="E56" s="15" t="inlineStr"/>
       <c r="F56" s="15" t="inlineStr"/>
-      <c r="G56" s="16" t="inlineStr"/>
+      <c r="G56" s="15" t="inlineStr"/>
       <c r="H56" s="16" t="inlineStr"/>
-      <c r="I56" s="15" t="inlineStr"/>
+      <c r="I56" s="16" t="inlineStr"/>
       <c r="J56" s="15" t="inlineStr"/>
-      <c r="K56" s="17" t="inlineStr"/>
+      <c r="K56" s="15" t="inlineStr"/>
       <c r="L56" s="17" t="inlineStr"/>
       <c r="M56" s="17" t="inlineStr"/>
       <c r="N56" s="17" t="inlineStr"/>
@@ -4064,6 +4157,7 @@
       <c r="AI56" s="17" t="inlineStr"/>
       <c r="AJ56" s="17" t="inlineStr"/>
       <c r="AK56" s="17" t="inlineStr"/>
+      <c r="AL56" s="17" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" s="15" t="inlineStr"/>
@@ -4072,11 +4166,11 @@
       <c r="D57" s="15" t="inlineStr"/>
       <c r="E57" s="15" t="inlineStr"/>
       <c r="F57" s="15" t="inlineStr"/>
-      <c r="G57" s="16" t="inlineStr"/>
+      <c r="G57" s="15" t="inlineStr"/>
       <c r="H57" s="16" t="inlineStr"/>
-      <c r="I57" s="15" t="inlineStr"/>
+      <c r="I57" s="16" t="inlineStr"/>
       <c r="J57" s="15" t="inlineStr"/>
-      <c r="K57" s="17" t="inlineStr"/>
+      <c r="K57" s="15" t="inlineStr"/>
       <c r="L57" s="17" t="inlineStr"/>
       <c r="M57" s="17" t="inlineStr"/>
       <c r="N57" s="17" t="inlineStr"/>
@@ -4103,6 +4197,7 @@
       <c r="AI57" s="17" t="inlineStr"/>
       <c r="AJ57" s="17" t="inlineStr"/>
       <c r="AK57" s="17" t="inlineStr"/>
+      <c r="AL57" s="17" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" s="15" t="inlineStr"/>
@@ -4111,11 +4206,11 @@
       <c r="D58" s="15" t="inlineStr"/>
       <c r="E58" s="15" t="inlineStr"/>
       <c r="F58" s="15" t="inlineStr"/>
-      <c r="G58" s="16" t="inlineStr"/>
+      <c r="G58" s="15" t="inlineStr"/>
       <c r="H58" s="16" t="inlineStr"/>
-      <c r="I58" s="15" t="inlineStr"/>
+      <c r="I58" s="16" t="inlineStr"/>
       <c r="J58" s="15" t="inlineStr"/>
-      <c r="K58" s="17" t="inlineStr"/>
+      <c r="K58" s="15" t="inlineStr"/>
       <c r="L58" s="17" t="inlineStr"/>
       <c r="M58" s="17" t="inlineStr"/>
       <c r="N58" s="17" t="inlineStr"/>
@@ -4142,6 +4237,7 @@
       <c r="AI58" s="17" t="inlineStr"/>
       <c r="AJ58" s="17" t="inlineStr"/>
       <c r="AK58" s="17" t="inlineStr"/>
+      <c r="AL58" s="17" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" s="15" t="inlineStr"/>
@@ -4150,11 +4246,11 @@
       <c r="D59" s="15" t="inlineStr"/>
       <c r="E59" s="15" t="inlineStr"/>
       <c r="F59" s="15" t="inlineStr"/>
-      <c r="G59" s="16" t="inlineStr"/>
+      <c r="G59" s="15" t="inlineStr"/>
       <c r="H59" s="16" t="inlineStr"/>
-      <c r="I59" s="15" t="inlineStr"/>
+      <c r="I59" s="16" t="inlineStr"/>
       <c r="J59" s="15" t="inlineStr"/>
-      <c r="K59" s="17" t="inlineStr"/>
+      <c r="K59" s="15" t="inlineStr"/>
       <c r="L59" s="17" t="inlineStr"/>
       <c r="M59" s="17" t="inlineStr"/>
       <c r="N59" s="17" t="inlineStr"/>
@@ -4181,6 +4277,7 @@
       <c r="AI59" s="17" t="inlineStr"/>
       <c r="AJ59" s="17" t="inlineStr"/>
       <c r="AK59" s="17" t="inlineStr"/>
+      <c r="AL59" s="17" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" s="15" t="inlineStr"/>
@@ -4189,11 +4286,11 @@
       <c r="D60" s="15" t="inlineStr"/>
       <c r="E60" s="15" t="inlineStr"/>
       <c r="F60" s="15" t="inlineStr"/>
-      <c r="G60" s="16" t="inlineStr"/>
+      <c r="G60" s="15" t="inlineStr"/>
       <c r="H60" s="16" t="inlineStr"/>
-      <c r="I60" s="15" t="inlineStr"/>
+      <c r="I60" s="16" t="inlineStr"/>
       <c r="J60" s="15" t="inlineStr"/>
-      <c r="K60" s="17" t="inlineStr"/>
+      <c r="K60" s="15" t="inlineStr"/>
       <c r="L60" s="17" t="inlineStr"/>
       <c r="M60" s="17" t="inlineStr"/>
       <c r="N60" s="17" t="inlineStr"/>
@@ -4220,6 +4317,7 @@
       <c r="AI60" s="17" t="inlineStr"/>
       <c r="AJ60" s="17" t="inlineStr"/>
       <c r="AK60" s="17" t="inlineStr"/>
+      <c r="AL60" s="17" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" s="15" t="inlineStr"/>
@@ -4228,11 +4326,11 @@
       <c r="D61" s="15" t="inlineStr"/>
       <c r="E61" s="15" t="inlineStr"/>
       <c r="F61" s="15" t="inlineStr"/>
-      <c r="G61" s="16" t="inlineStr"/>
+      <c r="G61" s="15" t="inlineStr"/>
       <c r="H61" s="16" t="inlineStr"/>
-      <c r="I61" s="15" t="inlineStr"/>
+      <c r="I61" s="16" t="inlineStr"/>
       <c r="J61" s="15" t="inlineStr"/>
-      <c r="K61" s="17" t="inlineStr"/>
+      <c r="K61" s="15" t="inlineStr"/>
       <c r="L61" s="17" t="inlineStr"/>
       <c r="M61" s="17" t="inlineStr"/>
       <c r="N61" s="17" t="inlineStr"/>
@@ -4259,6 +4357,7 @@
       <c r="AI61" s="17" t="inlineStr"/>
       <c r="AJ61" s="17" t="inlineStr"/>
       <c r="AK61" s="17" t="inlineStr"/>
+      <c r="AL61" s="17" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" s="15" t="inlineStr"/>
@@ -4267,11 +4366,11 @@
       <c r="D62" s="15" t="inlineStr"/>
       <c r="E62" s="15" t="inlineStr"/>
       <c r="F62" s="15" t="inlineStr"/>
-      <c r="G62" s="16" t="inlineStr"/>
+      <c r="G62" s="15" t="inlineStr"/>
       <c r="H62" s="16" t="inlineStr"/>
-      <c r="I62" s="15" t="inlineStr"/>
+      <c r="I62" s="16" t="inlineStr"/>
       <c r="J62" s="15" t="inlineStr"/>
-      <c r="K62" s="17" t="inlineStr"/>
+      <c r="K62" s="15" t="inlineStr"/>
       <c r="L62" s="17" t="inlineStr"/>
       <c r="M62" s="17" t="inlineStr"/>
       <c r="N62" s="17" t="inlineStr"/>
@@ -4298,6 +4397,7 @@
       <c r="AI62" s="17" t="inlineStr"/>
       <c r="AJ62" s="17" t="inlineStr"/>
       <c r="AK62" s="17" t="inlineStr"/>
+      <c r="AL62" s="17" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" s="15" t="inlineStr"/>
@@ -4306,11 +4406,11 @@
       <c r="D63" s="15" t="inlineStr"/>
       <c r="E63" s="15" t="inlineStr"/>
       <c r="F63" s="15" t="inlineStr"/>
-      <c r="G63" s="16" t="inlineStr"/>
+      <c r="G63" s="15" t="inlineStr"/>
       <c r="H63" s="16" t="inlineStr"/>
-      <c r="I63" s="15" t="inlineStr"/>
+      <c r="I63" s="16" t="inlineStr"/>
       <c r="J63" s="15" t="inlineStr"/>
-      <c r="K63" s="17" t="inlineStr"/>
+      <c r="K63" s="15" t="inlineStr"/>
       <c r="L63" s="17" t="inlineStr"/>
       <c r="M63" s="17" t="inlineStr"/>
       <c r="N63" s="17" t="inlineStr"/>
@@ -4337,6 +4437,7 @@
       <c r="AI63" s="17" t="inlineStr"/>
       <c r="AJ63" s="17" t="inlineStr"/>
       <c r="AK63" s="17" t="inlineStr"/>
+      <c r="AL63" s="17" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" s="15" t="inlineStr"/>
@@ -4345,11 +4446,11 @@
       <c r="D64" s="15" t="inlineStr"/>
       <c r="E64" s="15" t="inlineStr"/>
       <c r="F64" s="15" t="inlineStr"/>
-      <c r="G64" s="16" t="inlineStr"/>
+      <c r="G64" s="15" t="inlineStr"/>
       <c r="H64" s="16" t="inlineStr"/>
-      <c r="I64" s="15" t="inlineStr"/>
+      <c r="I64" s="16" t="inlineStr"/>
       <c r="J64" s="15" t="inlineStr"/>
-      <c r="K64" s="17" t="inlineStr"/>
+      <c r="K64" s="15" t="inlineStr"/>
       <c r="L64" s="17" t="inlineStr"/>
       <c r="M64" s="17" t="inlineStr"/>
       <c r="N64" s="17" t="inlineStr"/>
@@ -4376,6 +4477,7 @@
       <c r="AI64" s="17" t="inlineStr"/>
       <c r="AJ64" s="17" t="inlineStr"/>
       <c r="AK64" s="17" t="inlineStr"/>
+      <c r="AL64" s="17" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" s="15" t="inlineStr"/>
@@ -4384,11 +4486,11 @@
       <c r="D65" s="15" t="inlineStr"/>
       <c r="E65" s="15" t="inlineStr"/>
       <c r="F65" s="15" t="inlineStr"/>
-      <c r="G65" s="16" t="inlineStr"/>
+      <c r="G65" s="15" t="inlineStr"/>
       <c r="H65" s="16" t="inlineStr"/>
-      <c r="I65" s="15" t="inlineStr"/>
+      <c r="I65" s="16" t="inlineStr"/>
       <c r="J65" s="15" t="inlineStr"/>
-      <c r="K65" s="17" t="inlineStr"/>
+      <c r="K65" s="15" t="inlineStr"/>
       <c r="L65" s="17" t="inlineStr"/>
       <c r="M65" s="17" t="inlineStr"/>
       <c r="N65" s="17" t="inlineStr"/>
@@ -4415,6 +4517,7 @@
       <c r="AI65" s="17" t="inlineStr"/>
       <c r="AJ65" s="17" t="inlineStr"/>
       <c r="AK65" s="17" t="inlineStr"/>
+      <c r="AL65" s="17" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" s="15" t="inlineStr"/>
@@ -4423,11 +4526,11 @@
       <c r="D66" s="15" t="inlineStr"/>
       <c r="E66" s="15" t="inlineStr"/>
       <c r="F66" s="15" t="inlineStr"/>
-      <c r="G66" s="16" t="inlineStr"/>
+      <c r="G66" s="15" t="inlineStr"/>
       <c r="H66" s="16" t="inlineStr"/>
-      <c r="I66" s="15" t="inlineStr"/>
+      <c r="I66" s="16" t="inlineStr"/>
       <c r="J66" s="15" t="inlineStr"/>
-      <c r="K66" s="17" t="inlineStr"/>
+      <c r="K66" s="15" t="inlineStr"/>
       <c r="L66" s="17" t="inlineStr"/>
       <c r="M66" s="17" t="inlineStr"/>
       <c r="N66" s="17" t="inlineStr"/>
@@ -4454,6 +4557,7 @@
       <c r="AI66" s="17" t="inlineStr"/>
       <c r="AJ66" s="17" t="inlineStr"/>
       <c r="AK66" s="17" t="inlineStr"/>
+      <c r="AL66" s="17" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" s="15" t="inlineStr"/>
@@ -4462,11 +4566,11 @@
       <c r="D67" s="15" t="inlineStr"/>
       <c r="E67" s="15" t="inlineStr"/>
       <c r="F67" s="15" t="inlineStr"/>
-      <c r="G67" s="16" t="inlineStr"/>
+      <c r="G67" s="15" t="inlineStr"/>
       <c r="H67" s="16" t="inlineStr"/>
-      <c r="I67" s="15" t="inlineStr"/>
+      <c r="I67" s="16" t="inlineStr"/>
       <c r="J67" s="15" t="inlineStr"/>
-      <c r="K67" s="17" t="inlineStr"/>
+      <c r="K67" s="15" t="inlineStr"/>
       <c r="L67" s="17" t="inlineStr"/>
       <c r="M67" s="17" t="inlineStr"/>
       <c r="N67" s="17" t="inlineStr"/>
@@ -4493,6 +4597,7 @@
       <c r="AI67" s="17" t="inlineStr"/>
       <c r="AJ67" s="17" t="inlineStr"/>
       <c r="AK67" s="17" t="inlineStr"/>
+      <c r="AL67" s="17" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" s="15" t="inlineStr"/>
@@ -4501,11 +4606,11 @@
       <c r="D68" s="15" t="inlineStr"/>
       <c r="E68" s="15" t="inlineStr"/>
       <c r="F68" s="15" t="inlineStr"/>
-      <c r="G68" s="16" t="inlineStr"/>
+      <c r="G68" s="15" t="inlineStr"/>
       <c r="H68" s="16" t="inlineStr"/>
-      <c r="I68" s="15" t="inlineStr"/>
+      <c r="I68" s="16" t="inlineStr"/>
       <c r="J68" s="15" t="inlineStr"/>
-      <c r="K68" s="17" t="inlineStr"/>
+      <c r="K68" s="15" t="inlineStr"/>
       <c r="L68" s="17" t="inlineStr"/>
       <c r="M68" s="17" t="inlineStr"/>
       <c r="N68" s="17" t="inlineStr"/>
@@ -4532,6 +4637,7 @@
       <c r="AI68" s="17" t="inlineStr"/>
       <c r="AJ68" s="17" t="inlineStr"/>
       <c r="AK68" s="17" t="inlineStr"/>
+      <c r="AL68" s="17" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" s="15" t="inlineStr"/>
@@ -4540,11 +4646,11 @@
       <c r="D69" s="15" t="inlineStr"/>
       <c r="E69" s="15" t="inlineStr"/>
       <c r="F69" s="15" t="inlineStr"/>
-      <c r="G69" s="16" t="inlineStr"/>
+      <c r="G69" s="15" t="inlineStr"/>
       <c r="H69" s="16" t="inlineStr"/>
-      <c r="I69" s="15" t="inlineStr"/>
+      <c r="I69" s="16" t="inlineStr"/>
       <c r="J69" s="15" t="inlineStr"/>
-      <c r="K69" s="17" t="inlineStr"/>
+      <c r="K69" s="15" t="inlineStr"/>
       <c r="L69" s="17" t="inlineStr"/>
       <c r="M69" s="17" t="inlineStr"/>
       <c r="N69" s="17" t="inlineStr"/>
@@ -4571,6 +4677,7 @@
       <c r="AI69" s="17" t="inlineStr"/>
       <c r="AJ69" s="17" t="inlineStr"/>
       <c r="AK69" s="17" t="inlineStr"/>
+      <c r="AL69" s="17" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" s="15" t="inlineStr"/>
@@ -4579,11 +4686,11 @@
       <c r="D70" s="15" t="inlineStr"/>
       <c r="E70" s="15" t="inlineStr"/>
       <c r="F70" s="15" t="inlineStr"/>
-      <c r="G70" s="16" t="inlineStr"/>
+      <c r="G70" s="15" t="inlineStr"/>
       <c r="H70" s="16" t="inlineStr"/>
-      <c r="I70" s="15" t="inlineStr"/>
+      <c r="I70" s="16" t="inlineStr"/>
       <c r="J70" s="15" t="inlineStr"/>
-      <c r="K70" s="17" t="inlineStr"/>
+      <c r="K70" s="15" t="inlineStr"/>
       <c r="L70" s="17" t="inlineStr"/>
       <c r="M70" s="17" t="inlineStr"/>
       <c r="N70" s="17" t="inlineStr"/>
@@ -4610,6 +4717,7 @@
       <c r="AI70" s="17" t="inlineStr"/>
       <c r="AJ70" s="17" t="inlineStr"/>
       <c r="AK70" s="17" t="inlineStr"/>
+      <c r="AL70" s="17" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" s="15" t="inlineStr"/>
@@ -4618,11 +4726,11 @@
       <c r="D71" s="15" t="inlineStr"/>
       <c r="E71" s="15" t="inlineStr"/>
       <c r="F71" s="15" t="inlineStr"/>
-      <c r="G71" s="16" t="inlineStr"/>
+      <c r="G71" s="15" t="inlineStr"/>
       <c r="H71" s="16" t="inlineStr"/>
-      <c r="I71" s="15" t="inlineStr"/>
+      <c r="I71" s="16" t="inlineStr"/>
       <c r="J71" s="15" t="inlineStr"/>
-      <c r="K71" s="17" t="inlineStr"/>
+      <c r="K71" s="15" t="inlineStr"/>
       <c r="L71" s="17" t="inlineStr"/>
       <c r="M71" s="17" t="inlineStr"/>
       <c r="N71" s="17" t="inlineStr"/>
@@ -4649,6 +4757,7 @@
       <c r="AI71" s="17" t="inlineStr"/>
       <c r="AJ71" s="17" t="inlineStr"/>
       <c r="AK71" s="17" t="inlineStr"/>
+      <c r="AL71" s="17" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" s="15" t="inlineStr"/>
@@ -4657,11 +4766,11 @@
       <c r="D72" s="15" t="inlineStr"/>
       <c r="E72" s="15" t="inlineStr"/>
       <c r="F72" s="15" t="inlineStr"/>
-      <c r="G72" s="16" t="inlineStr"/>
+      <c r="G72" s="15" t="inlineStr"/>
       <c r="H72" s="16" t="inlineStr"/>
-      <c r="I72" s="15" t="inlineStr"/>
+      <c r="I72" s="16" t="inlineStr"/>
       <c r="J72" s="15" t="inlineStr"/>
-      <c r="K72" s="17" t="inlineStr"/>
+      <c r="K72" s="15" t="inlineStr"/>
       <c r="L72" s="17" t="inlineStr"/>
       <c r="M72" s="17" t="inlineStr"/>
       <c r="N72" s="17" t="inlineStr"/>
@@ -4688,6 +4797,7 @@
       <c r="AI72" s="17" t="inlineStr"/>
       <c r="AJ72" s="17" t="inlineStr"/>
       <c r="AK72" s="17" t="inlineStr"/>
+      <c r="AL72" s="17" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" s="15" t="inlineStr"/>
@@ -4696,11 +4806,11 @@
       <c r="D73" s="15" t="inlineStr"/>
       <c r="E73" s="15" t="inlineStr"/>
       <c r="F73" s="15" t="inlineStr"/>
-      <c r="G73" s="16" t="inlineStr"/>
+      <c r="G73" s="15" t="inlineStr"/>
       <c r="H73" s="16" t="inlineStr"/>
-      <c r="I73" s="15" t="inlineStr"/>
+      <c r="I73" s="16" t="inlineStr"/>
       <c r="J73" s="15" t="inlineStr"/>
-      <c r="K73" s="17" t="inlineStr"/>
+      <c r="K73" s="15" t="inlineStr"/>
       <c r="L73" s="17" t="inlineStr"/>
       <c r="M73" s="17" t="inlineStr"/>
       <c r="N73" s="17" t="inlineStr"/>
@@ -4727,6 +4837,7 @@
       <c r="AI73" s="17" t="inlineStr"/>
       <c r="AJ73" s="17" t="inlineStr"/>
       <c r="AK73" s="17" t="inlineStr"/>
+      <c r="AL73" s="17" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" s="15" t="inlineStr"/>
@@ -4735,11 +4846,11 @@
       <c r="D74" s="15" t="inlineStr"/>
       <c r="E74" s="15" t="inlineStr"/>
       <c r="F74" s="15" t="inlineStr"/>
-      <c r="G74" s="16" t="inlineStr"/>
+      <c r="G74" s="15" t="inlineStr"/>
       <c r="H74" s="16" t="inlineStr"/>
-      <c r="I74" s="15" t="inlineStr"/>
+      <c r="I74" s="16" t="inlineStr"/>
       <c r="J74" s="15" t="inlineStr"/>
-      <c r="K74" s="17" t="inlineStr"/>
+      <c r="K74" s="15" t="inlineStr"/>
       <c r="L74" s="17" t="inlineStr"/>
       <c r="M74" s="17" t="inlineStr"/>
       <c r="N74" s="17" t="inlineStr"/>
@@ -4766,6 +4877,7 @@
       <c r="AI74" s="17" t="inlineStr"/>
       <c r="AJ74" s="17" t="inlineStr"/>
       <c r="AK74" s="17" t="inlineStr"/>
+      <c r="AL74" s="17" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" s="15" t="inlineStr"/>
@@ -4774,11 +4886,11 @@
       <c r="D75" s="15" t="inlineStr"/>
       <c r="E75" s="15" t="inlineStr"/>
       <c r="F75" s="15" t="inlineStr"/>
-      <c r="G75" s="16" t="inlineStr"/>
+      <c r="G75" s="15" t="inlineStr"/>
       <c r="H75" s="16" t="inlineStr"/>
-      <c r="I75" s="15" t="inlineStr"/>
+      <c r="I75" s="16" t="inlineStr"/>
       <c r="J75" s="15" t="inlineStr"/>
-      <c r="K75" s="17" t="inlineStr"/>
+      <c r="K75" s="15" t="inlineStr"/>
       <c r="L75" s="17" t="inlineStr"/>
       <c r="M75" s="17" t="inlineStr"/>
       <c r="N75" s="17" t="inlineStr"/>
@@ -4805,6 +4917,7 @@
       <c r="AI75" s="17" t="inlineStr"/>
       <c r="AJ75" s="17" t="inlineStr"/>
       <c r="AK75" s="17" t="inlineStr"/>
+      <c r="AL75" s="17" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" s="15" t="inlineStr"/>
@@ -4813,11 +4926,11 @@
       <c r="D76" s="15" t="inlineStr"/>
       <c r="E76" s="15" t="inlineStr"/>
       <c r="F76" s="15" t="inlineStr"/>
-      <c r="G76" s="16" t="inlineStr"/>
+      <c r="G76" s="15" t="inlineStr"/>
       <c r="H76" s="16" t="inlineStr"/>
-      <c r="I76" s="15" t="inlineStr"/>
+      <c r="I76" s="16" t="inlineStr"/>
       <c r="J76" s="15" t="inlineStr"/>
-      <c r="K76" s="17" t="inlineStr"/>
+      <c r="K76" s="15" t="inlineStr"/>
       <c r="L76" s="17" t="inlineStr"/>
       <c r="M76" s="17" t="inlineStr"/>
       <c r="N76" s="17" t="inlineStr"/>
@@ -4844,6 +4957,7 @@
       <c r="AI76" s="17" t="inlineStr"/>
       <c r="AJ76" s="17" t="inlineStr"/>
       <c r="AK76" s="17" t="inlineStr"/>
+      <c r="AL76" s="17" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" s="15" t="inlineStr"/>
@@ -4852,11 +4966,11 @@
       <c r="D77" s="15" t="inlineStr"/>
       <c r="E77" s="15" t="inlineStr"/>
       <c r="F77" s="15" t="inlineStr"/>
-      <c r="G77" s="16" t="inlineStr"/>
+      <c r="G77" s="15" t="inlineStr"/>
       <c r="H77" s="16" t="inlineStr"/>
-      <c r="I77" s="15" t="inlineStr"/>
+      <c r="I77" s="16" t="inlineStr"/>
       <c r="J77" s="15" t="inlineStr"/>
-      <c r="K77" s="17" t="inlineStr"/>
+      <c r="K77" s="15" t="inlineStr"/>
       <c r="L77" s="17" t="inlineStr"/>
       <c r="M77" s="17" t="inlineStr"/>
       <c r="N77" s="17" t="inlineStr"/>
@@ -4883,6 +4997,7 @@
       <c r="AI77" s="17" t="inlineStr"/>
       <c r="AJ77" s="17" t="inlineStr"/>
       <c r="AK77" s="17" t="inlineStr"/>
+      <c r="AL77" s="17" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" s="15" t="inlineStr"/>
@@ -4891,11 +5006,11 @@
       <c r="D78" s="15" t="inlineStr"/>
       <c r="E78" s="15" t="inlineStr"/>
       <c r="F78" s="15" t="inlineStr"/>
-      <c r="G78" s="16" t="inlineStr"/>
+      <c r="G78" s="15" t="inlineStr"/>
       <c r="H78" s="16" t="inlineStr"/>
-      <c r="I78" s="15" t="inlineStr"/>
+      <c r="I78" s="16" t="inlineStr"/>
       <c r="J78" s="15" t="inlineStr"/>
-      <c r="K78" s="17" t="inlineStr"/>
+      <c r="K78" s="15" t="inlineStr"/>
       <c r="L78" s="17" t="inlineStr"/>
       <c r="M78" s="17" t="inlineStr"/>
       <c r="N78" s="17" t="inlineStr"/>
@@ -4922,6 +5037,7 @@
       <c r="AI78" s="17" t="inlineStr"/>
       <c r="AJ78" s="17" t="inlineStr"/>
       <c r="AK78" s="17" t="inlineStr"/>
+      <c r="AL78" s="17" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" s="15" t="inlineStr"/>
@@ -4930,11 +5046,11 @@
       <c r="D79" s="15" t="inlineStr"/>
       <c r="E79" s="15" t="inlineStr"/>
       <c r="F79" s="15" t="inlineStr"/>
-      <c r="G79" s="16" t="inlineStr"/>
+      <c r="G79" s="15" t="inlineStr"/>
       <c r="H79" s="16" t="inlineStr"/>
-      <c r="I79" s="15" t="inlineStr"/>
+      <c r="I79" s="16" t="inlineStr"/>
       <c r="J79" s="15" t="inlineStr"/>
-      <c r="K79" s="17" t="inlineStr"/>
+      <c r="K79" s="15" t="inlineStr"/>
       <c r="L79" s="17" t="inlineStr"/>
       <c r="M79" s="17" t="inlineStr"/>
       <c r="N79" s="17" t="inlineStr"/>
@@ -4961,6 +5077,7 @@
       <c r="AI79" s="17" t="inlineStr"/>
       <c r="AJ79" s="17" t="inlineStr"/>
       <c r="AK79" s="17" t="inlineStr"/>
+      <c r="AL79" s="17" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" s="15" t="inlineStr"/>
@@ -4969,11 +5086,11 @@
       <c r="D80" s="15" t="inlineStr"/>
       <c r="E80" s="15" t="inlineStr"/>
       <c r="F80" s="15" t="inlineStr"/>
-      <c r="G80" s="16" t="inlineStr"/>
+      <c r="G80" s="15" t="inlineStr"/>
       <c r="H80" s="16" t="inlineStr"/>
-      <c r="I80" s="15" t="inlineStr"/>
+      <c r="I80" s="16" t="inlineStr"/>
       <c r="J80" s="15" t="inlineStr"/>
-      <c r="K80" s="17" t="inlineStr"/>
+      <c r="K80" s="15" t="inlineStr"/>
       <c r="L80" s="17" t="inlineStr"/>
       <c r="M80" s="17" t="inlineStr"/>
       <c r="N80" s="17" t="inlineStr"/>
@@ -5000,6 +5117,7 @@
       <c r="AI80" s="17" t="inlineStr"/>
       <c r="AJ80" s="17" t="inlineStr"/>
       <c r="AK80" s="17" t="inlineStr"/>
+      <c r="AL80" s="17" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" s="15" t="inlineStr"/>
@@ -5008,11 +5126,11 @@
       <c r="D81" s="15" t="inlineStr"/>
       <c r="E81" s="15" t="inlineStr"/>
       <c r="F81" s="15" t="inlineStr"/>
-      <c r="G81" s="16" t="inlineStr"/>
+      <c r="G81" s="15" t="inlineStr"/>
       <c r="H81" s="16" t="inlineStr"/>
-      <c r="I81" s="15" t="inlineStr"/>
+      <c r="I81" s="16" t="inlineStr"/>
       <c r="J81" s="15" t="inlineStr"/>
-      <c r="K81" s="17" t="inlineStr"/>
+      <c r="K81" s="15" t="inlineStr"/>
       <c r="L81" s="17" t="inlineStr"/>
       <c r="M81" s="17" t="inlineStr"/>
       <c r="N81" s="17" t="inlineStr"/>
@@ -5039,6 +5157,7 @@
       <c r="AI81" s="17" t="inlineStr"/>
       <c r="AJ81" s="17" t="inlineStr"/>
       <c r="AK81" s="17" t="inlineStr"/>
+      <c r="AL81" s="17" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" s="15" t="inlineStr"/>
@@ -5047,11 +5166,11 @@
       <c r="D82" s="15" t="inlineStr"/>
       <c r="E82" s="15" t="inlineStr"/>
       <c r="F82" s="15" t="inlineStr"/>
-      <c r="G82" s="16" t="inlineStr"/>
+      <c r="G82" s="15" t="inlineStr"/>
       <c r="H82" s="16" t="inlineStr"/>
-      <c r="I82" s="15" t="inlineStr"/>
+      <c r="I82" s="16" t="inlineStr"/>
       <c r="J82" s="15" t="inlineStr"/>
-      <c r="K82" s="17" t="inlineStr"/>
+      <c r="K82" s="15" t="inlineStr"/>
       <c r="L82" s="17" t="inlineStr"/>
       <c r="M82" s="17" t="inlineStr"/>
       <c r="N82" s="17" t="inlineStr"/>
@@ -5078,6 +5197,7 @@
       <c r="AI82" s="17" t="inlineStr"/>
       <c r="AJ82" s="17" t="inlineStr"/>
       <c r="AK82" s="17" t="inlineStr"/>
+      <c r="AL82" s="17" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" s="15" t="inlineStr"/>
@@ -5086,11 +5206,11 @@
       <c r="D83" s="15" t="inlineStr"/>
       <c r="E83" s="15" t="inlineStr"/>
       <c r="F83" s="15" t="inlineStr"/>
-      <c r="G83" s="16" t="inlineStr"/>
+      <c r="G83" s="15" t="inlineStr"/>
       <c r="H83" s="16" t="inlineStr"/>
-      <c r="I83" s="15" t="inlineStr"/>
+      <c r="I83" s="16" t="inlineStr"/>
       <c r="J83" s="15" t="inlineStr"/>
-      <c r="K83" s="17" t="inlineStr"/>
+      <c r="K83" s="15" t="inlineStr"/>
       <c r="L83" s="17" t="inlineStr"/>
       <c r="M83" s="17" t="inlineStr"/>
       <c r="N83" s="17" t="inlineStr"/>
@@ -5117,6 +5237,7 @@
       <c r="AI83" s="17" t="inlineStr"/>
       <c r="AJ83" s="17" t="inlineStr"/>
       <c r="AK83" s="17" t="inlineStr"/>
+      <c r="AL83" s="17" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" s="15" t="inlineStr"/>
@@ -5125,11 +5246,11 @@
       <c r="D84" s="15" t="inlineStr"/>
       <c r="E84" s="15" t="inlineStr"/>
       <c r="F84" s="15" t="inlineStr"/>
-      <c r="G84" s="16" t="inlineStr"/>
+      <c r="G84" s="15" t="inlineStr"/>
       <c r="H84" s="16" t="inlineStr"/>
-      <c r="I84" s="15" t="inlineStr"/>
+      <c r="I84" s="16" t="inlineStr"/>
       <c r="J84" s="15" t="inlineStr"/>
-      <c r="K84" s="17" t="inlineStr"/>
+      <c r="K84" s="15" t="inlineStr"/>
       <c r="L84" s="17" t="inlineStr"/>
       <c r="M84" s="17" t="inlineStr"/>
       <c r="N84" s="17" t="inlineStr"/>
@@ -5156,6 +5277,7 @@
       <c r="AI84" s="17" t="inlineStr"/>
       <c r="AJ84" s="17" t="inlineStr"/>
       <c r="AK84" s="17" t="inlineStr"/>
+      <c r="AL84" s="17" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" s="15" t="inlineStr"/>
@@ -5164,11 +5286,11 @@
       <c r="D85" s="15" t="inlineStr"/>
       <c r="E85" s="15" t="inlineStr"/>
       <c r="F85" s="15" t="inlineStr"/>
-      <c r="G85" s="16" t="inlineStr"/>
+      <c r="G85" s="15" t="inlineStr"/>
       <c r="H85" s="16" t="inlineStr"/>
-      <c r="I85" s="15" t="inlineStr"/>
+      <c r="I85" s="16" t="inlineStr"/>
       <c r="J85" s="15" t="inlineStr"/>
-      <c r="K85" s="17" t="inlineStr"/>
+      <c r="K85" s="15" t="inlineStr"/>
       <c r="L85" s="17" t="inlineStr"/>
       <c r="M85" s="17" t="inlineStr"/>
       <c r="N85" s="17" t="inlineStr"/>
@@ -5195,6 +5317,7 @@
       <c r="AI85" s="17" t="inlineStr"/>
       <c r="AJ85" s="17" t="inlineStr"/>
       <c r="AK85" s="17" t="inlineStr"/>
+      <c r="AL85" s="17" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" s="15" t="inlineStr"/>
@@ -5203,11 +5326,11 @@
       <c r="D86" s="15" t="inlineStr"/>
       <c r="E86" s="15" t="inlineStr"/>
       <c r="F86" s="15" t="inlineStr"/>
-      <c r="G86" s="16" t="inlineStr"/>
+      <c r="G86" s="15" t="inlineStr"/>
       <c r="H86" s="16" t="inlineStr"/>
-      <c r="I86" s="15" t="inlineStr"/>
+      <c r="I86" s="16" t="inlineStr"/>
       <c r="J86" s="15" t="inlineStr"/>
-      <c r="K86" s="17" t="inlineStr"/>
+      <c r="K86" s="15" t="inlineStr"/>
       <c r="L86" s="17" t="inlineStr"/>
       <c r="M86" s="17" t="inlineStr"/>
       <c r="N86" s="17" t="inlineStr"/>
@@ -5234,6 +5357,7 @@
       <c r="AI86" s="17" t="inlineStr"/>
       <c r="AJ86" s="17" t="inlineStr"/>
       <c r="AK86" s="17" t="inlineStr"/>
+      <c r="AL86" s="17" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" s="15" t="inlineStr"/>
@@ -5242,11 +5366,11 @@
       <c r="D87" s="15" t="inlineStr"/>
       <c r="E87" s="15" t="inlineStr"/>
       <c r="F87" s="15" t="inlineStr"/>
-      <c r="G87" s="16" t="inlineStr"/>
+      <c r="G87" s="15" t="inlineStr"/>
       <c r="H87" s="16" t="inlineStr"/>
-      <c r="I87" s="15" t="inlineStr"/>
+      <c r="I87" s="16" t="inlineStr"/>
       <c r="J87" s="15" t="inlineStr"/>
-      <c r="K87" s="17" t="inlineStr"/>
+      <c r="K87" s="15" t="inlineStr"/>
       <c r="L87" s="17" t="inlineStr"/>
       <c r="M87" s="17" t="inlineStr"/>
       <c r="N87" s="17" t="inlineStr"/>
@@ -5273,6 +5397,7 @@
       <c r="AI87" s="17" t="inlineStr"/>
       <c r="AJ87" s="17" t="inlineStr"/>
       <c r="AK87" s="17" t="inlineStr"/>
+      <c r="AL87" s="17" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" s="15" t="inlineStr"/>
@@ -5281,11 +5406,11 @@
       <c r="D88" s="15" t="inlineStr"/>
       <c r="E88" s="15" t="inlineStr"/>
       <c r="F88" s="15" t="inlineStr"/>
-      <c r="G88" s="16" t="inlineStr"/>
+      <c r="G88" s="15" t="inlineStr"/>
       <c r="H88" s="16" t="inlineStr"/>
-      <c r="I88" s="15" t="inlineStr"/>
+      <c r="I88" s="16" t="inlineStr"/>
       <c r="J88" s="15" t="inlineStr"/>
-      <c r="K88" s="17" t="inlineStr"/>
+      <c r="K88" s="15" t="inlineStr"/>
       <c r="L88" s="17" t="inlineStr"/>
       <c r="M88" s="17" t="inlineStr"/>
       <c r="N88" s="17" t="inlineStr"/>
@@ -5312,6 +5437,7 @@
       <c r="AI88" s="17" t="inlineStr"/>
       <c r="AJ88" s="17" t="inlineStr"/>
       <c r="AK88" s="17" t="inlineStr"/>
+      <c r="AL88" s="17" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" s="15" t="inlineStr"/>
@@ -5320,11 +5446,11 @@
       <c r="D89" s="15" t="inlineStr"/>
       <c r="E89" s="15" t="inlineStr"/>
       <c r="F89" s="15" t="inlineStr"/>
-      <c r="G89" s="16" t="inlineStr"/>
+      <c r="G89" s="15" t="inlineStr"/>
       <c r="H89" s="16" t="inlineStr"/>
-      <c r="I89" s="15" t="inlineStr"/>
+      <c r="I89" s="16" t="inlineStr"/>
       <c r="J89" s="15" t="inlineStr"/>
-      <c r="K89" s="17" t="inlineStr"/>
+      <c r="K89" s="15" t="inlineStr"/>
       <c r="L89" s="17" t="inlineStr"/>
       <c r="M89" s="17" t="inlineStr"/>
       <c r="N89" s="17" t="inlineStr"/>
@@ -5351,6 +5477,7 @@
       <c r="AI89" s="17" t="inlineStr"/>
       <c r="AJ89" s="17" t="inlineStr"/>
       <c r="AK89" s="17" t="inlineStr"/>
+      <c r="AL89" s="17" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" s="15" t="inlineStr"/>
@@ -5359,11 +5486,11 @@
       <c r="D90" s="15" t="inlineStr"/>
       <c r="E90" s="15" t="inlineStr"/>
       <c r="F90" s="15" t="inlineStr"/>
-      <c r="G90" s="16" t="inlineStr"/>
+      <c r="G90" s="15" t="inlineStr"/>
       <c r="H90" s="16" t="inlineStr"/>
-      <c r="I90" s="15" t="inlineStr"/>
+      <c r="I90" s="16" t="inlineStr"/>
       <c r="J90" s="15" t="inlineStr"/>
-      <c r="K90" s="17" t="inlineStr"/>
+      <c r="K90" s="15" t="inlineStr"/>
       <c r="L90" s="17" t="inlineStr"/>
       <c r="M90" s="17" t="inlineStr"/>
       <c r="N90" s="17" t="inlineStr"/>
@@ -5390,6 +5517,7 @@
       <c r="AI90" s="17" t="inlineStr"/>
       <c r="AJ90" s="17" t="inlineStr"/>
       <c r="AK90" s="17" t="inlineStr"/>
+      <c r="AL90" s="17" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" s="15" t="inlineStr"/>
@@ -5398,11 +5526,11 @@
       <c r="D91" s="15" t="inlineStr"/>
       <c r="E91" s="15" t="inlineStr"/>
       <c r="F91" s="15" t="inlineStr"/>
-      <c r="G91" s="16" t="inlineStr"/>
+      <c r="G91" s="15" t="inlineStr"/>
       <c r="H91" s="16" t="inlineStr"/>
-      <c r="I91" s="15" t="inlineStr"/>
+      <c r="I91" s="16" t="inlineStr"/>
       <c r="J91" s="15" t="inlineStr"/>
-      <c r="K91" s="17" t="inlineStr"/>
+      <c r="K91" s="15" t="inlineStr"/>
       <c r="L91" s="17" t="inlineStr"/>
       <c r="M91" s="17" t="inlineStr"/>
       <c r="N91" s="17" t="inlineStr"/>
@@ -5429,6 +5557,7 @@
       <c r="AI91" s="17" t="inlineStr"/>
       <c r="AJ91" s="17" t="inlineStr"/>
       <c r="AK91" s="17" t="inlineStr"/>
+      <c r="AL91" s="17" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" s="15" t="inlineStr"/>
@@ -5437,11 +5566,11 @@
       <c r="D92" s="15" t="inlineStr"/>
       <c r="E92" s="15" t="inlineStr"/>
       <c r="F92" s="15" t="inlineStr"/>
-      <c r="G92" s="16" t="inlineStr"/>
+      <c r="G92" s="15" t="inlineStr"/>
       <c r="H92" s="16" t="inlineStr"/>
-      <c r="I92" s="15" t="inlineStr"/>
+      <c r="I92" s="16" t="inlineStr"/>
       <c r="J92" s="15" t="inlineStr"/>
-      <c r="K92" s="17" t="inlineStr"/>
+      <c r="K92" s="15" t="inlineStr"/>
       <c r="L92" s="17" t="inlineStr"/>
       <c r="M92" s="17" t="inlineStr"/>
       <c r="N92" s="17" t="inlineStr"/>
@@ -5468,6 +5597,7 @@
       <c r="AI92" s="17" t="inlineStr"/>
       <c r="AJ92" s="17" t="inlineStr"/>
       <c r="AK92" s="17" t="inlineStr"/>
+      <c r="AL92" s="17" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" s="15" t="inlineStr"/>
@@ -5476,11 +5606,11 @@
       <c r="D93" s="15" t="inlineStr"/>
       <c r="E93" s="15" t="inlineStr"/>
       <c r="F93" s="15" t="inlineStr"/>
-      <c r="G93" s="16" t="inlineStr"/>
+      <c r="G93" s="15" t="inlineStr"/>
       <c r="H93" s="16" t="inlineStr"/>
-      <c r="I93" s="15" t="inlineStr"/>
+      <c r="I93" s="16" t="inlineStr"/>
       <c r="J93" s="15" t="inlineStr"/>
-      <c r="K93" s="17" t="inlineStr"/>
+      <c r="K93" s="15" t="inlineStr"/>
       <c r="L93" s="17" t="inlineStr"/>
       <c r="M93" s="17" t="inlineStr"/>
       <c r="N93" s="17" t="inlineStr"/>
@@ -5507,6 +5637,7 @@
       <c r="AI93" s="17" t="inlineStr"/>
       <c r="AJ93" s="17" t="inlineStr"/>
       <c r="AK93" s="17" t="inlineStr"/>
+      <c r="AL93" s="17" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" s="15" t="inlineStr"/>
@@ -5515,11 +5646,11 @@
       <c r="D94" s="15" t="inlineStr"/>
       <c r="E94" s="15" t="inlineStr"/>
       <c r="F94" s="15" t="inlineStr"/>
-      <c r="G94" s="16" t="inlineStr"/>
+      <c r="G94" s="15" t="inlineStr"/>
       <c r="H94" s="16" t="inlineStr"/>
-      <c r="I94" s="15" t="inlineStr"/>
+      <c r="I94" s="16" t="inlineStr"/>
       <c r="J94" s="15" t="inlineStr"/>
-      <c r="K94" s="17" t="inlineStr"/>
+      <c r="K94" s="15" t="inlineStr"/>
       <c r="L94" s="17" t="inlineStr"/>
       <c r="M94" s="17" t="inlineStr"/>
       <c r="N94" s="17" t="inlineStr"/>
@@ -5546,6 +5677,7 @@
       <c r="AI94" s="17" t="inlineStr"/>
       <c r="AJ94" s="17" t="inlineStr"/>
       <c r="AK94" s="17" t="inlineStr"/>
+      <c r="AL94" s="17" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" s="15" t="inlineStr"/>
@@ -5554,11 +5686,11 @@
       <c r="D95" s="15" t="inlineStr"/>
       <c r="E95" s="15" t="inlineStr"/>
       <c r="F95" s="15" t="inlineStr"/>
-      <c r="G95" s="16" t="inlineStr"/>
+      <c r="G95" s="15" t="inlineStr"/>
       <c r="H95" s="16" t="inlineStr"/>
-      <c r="I95" s="15" t="inlineStr"/>
+      <c r="I95" s="16" t="inlineStr"/>
       <c r="J95" s="15" t="inlineStr"/>
-      <c r="K95" s="17" t="inlineStr"/>
+      <c r="K95" s="15" t="inlineStr"/>
       <c r="L95" s="17" t="inlineStr"/>
       <c r="M95" s="17" t="inlineStr"/>
       <c r="N95" s="17" t="inlineStr"/>
@@ -5585,6 +5717,7 @@
       <c r="AI95" s="17" t="inlineStr"/>
       <c r="AJ95" s="17" t="inlineStr"/>
       <c r="AK95" s="17" t="inlineStr"/>
+      <c r="AL95" s="17" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" s="15" t="inlineStr"/>
@@ -5593,11 +5726,11 @@
       <c r="D96" s="15" t="inlineStr"/>
       <c r="E96" s="15" t="inlineStr"/>
       <c r="F96" s="15" t="inlineStr"/>
-      <c r="G96" s="16" t="inlineStr"/>
+      <c r="G96" s="15" t="inlineStr"/>
       <c r="H96" s="16" t="inlineStr"/>
-      <c r="I96" s="15" t="inlineStr"/>
+      <c r="I96" s="16" t="inlineStr"/>
       <c r="J96" s="15" t="inlineStr"/>
-      <c r="K96" s="17" t="inlineStr"/>
+      <c r="K96" s="15" t="inlineStr"/>
       <c r="L96" s="17" t="inlineStr"/>
       <c r="M96" s="17" t="inlineStr"/>
       <c r="N96" s="17" t="inlineStr"/>
@@ -5624,6 +5757,7 @@
       <c r="AI96" s="17" t="inlineStr"/>
       <c r="AJ96" s="17" t="inlineStr"/>
       <c r="AK96" s="17" t="inlineStr"/>
+      <c r="AL96" s="17" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" s="15" t="inlineStr"/>
@@ -5632,11 +5766,11 @@
       <c r="D97" s="15" t="inlineStr"/>
       <c r="E97" s="15" t="inlineStr"/>
       <c r="F97" s="15" t="inlineStr"/>
-      <c r="G97" s="16" t="inlineStr"/>
+      <c r="G97" s="15" t="inlineStr"/>
       <c r="H97" s="16" t="inlineStr"/>
-      <c r="I97" s="15" t="inlineStr"/>
+      <c r="I97" s="16" t="inlineStr"/>
       <c r="J97" s="15" t="inlineStr"/>
-      <c r="K97" s="17" t="inlineStr"/>
+      <c r="K97" s="15" t="inlineStr"/>
       <c r="L97" s="17" t="inlineStr"/>
       <c r="M97" s="17" t="inlineStr"/>
       <c r="N97" s="17" t="inlineStr"/>
@@ -5663,6 +5797,7 @@
       <c r="AI97" s="17" t="inlineStr"/>
       <c r="AJ97" s="17" t="inlineStr"/>
       <c r="AK97" s="17" t="inlineStr"/>
+      <c r="AL97" s="17" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" s="15" t="inlineStr"/>
@@ -5671,11 +5806,11 @@
       <c r="D98" s="15" t="inlineStr"/>
       <c r="E98" s="15" t="inlineStr"/>
       <c r="F98" s="15" t="inlineStr"/>
-      <c r="G98" s="16" t="inlineStr"/>
+      <c r="G98" s="15" t="inlineStr"/>
       <c r="H98" s="16" t="inlineStr"/>
-      <c r="I98" s="15" t="inlineStr"/>
+      <c r="I98" s="16" t="inlineStr"/>
       <c r="J98" s="15" t="inlineStr"/>
-      <c r="K98" s="17" t="inlineStr"/>
+      <c r="K98" s="15" t="inlineStr"/>
       <c r="L98" s="17" t="inlineStr"/>
       <c r="M98" s="17" t="inlineStr"/>
       <c r="N98" s="17" t="inlineStr"/>
@@ -5702,6 +5837,7 @@
       <c r="AI98" s="17" t="inlineStr"/>
       <c r="AJ98" s="17" t="inlineStr"/>
       <c r="AK98" s="17" t="inlineStr"/>
+      <c r="AL98" s="17" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" s="15" t="inlineStr"/>
@@ -5710,11 +5846,11 @@
       <c r="D99" s="15" t="inlineStr"/>
       <c r="E99" s="15" t="inlineStr"/>
       <c r="F99" s="15" t="inlineStr"/>
-      <c r="G99" s="16" t="inlineStr"/>
+      <c r="G99" s="15" t="inlineStr"/>
       <c r="H99" s="16" t="inlineStr"/>
-      <c r="I99" s="15" t="inlineStr"/>
+      <c r="I99" s="16" t="inlineStr"/>
       <c r="J99" s="15" t="inlineStr"/>
-      <c r="K99" s="17" t="inlineStr"/>
+      <c r="K99" s="15" t="inlineStr"/>
       <c r="L99" s="17" t="inlineStr"/>
       <c r="M99" s="17" t="inlineStr"/>
       <c r="N99" s="17" t="inlineStr"/>
@@ -5741,6 +5877,7 @@
       <c r="AI99" s="17" t="inlineStr"/>
       <c r="AJ99" s="17" t="inlineStr"/>
       <c r="AK99" s="17" t="inlineStr"/>
+      <c r="AL99" s="17" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" s="15" t="inlineStr"/>
@@ -5749,11 +5886,11 @@
       <c r="D100" s="15" t="inlineStr"/>
       <c r="E100" s="15" t="inlineStr"/>
       <c r="F100" s="15" t="inlineStr"/>
-      <c r="G100" s="16" t="inlineStr"/>
+      <c r="G100" s="15" t="inlineStr"/>
       <c r="H100" s="16" t="inlineStr"/>
-      <c r="I100" s="15" t="inlineStr"/>
+      <c r="I100" s="16" t="inlineStr"/>
       <c r="J100" s="15" t="inlineStr"/>
-      <c r="K100" s="17" t="inlineStr"/>
+      <c r="K100" s="15" t="inlineStr"/>
       <c r="L100" s="17" t="inlineStr"/>
       <c r="M100" s="17" t="inlineStr"/>
       <c r="N100" s="17" t="inlineStr"/>
@@ -5780,6 +5917,7 @@
       <c r="AI100" s="17" t="inlineStr"/>
       <c r="AJ100" s="17" t="inlineStr"/>
       <c r="AK100" s="17" t="inlineStr"/>
+      <c r="AL100" s="17" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" s="15" t="inlineStr"/>
@@ -5788,11 +5926,11 @@
       <c r="D101" s="15" t="inlineStr"/>
       <c r="E101" s="15" t="inlineStr"/>
       <c r="F101" s="15" t="inlineStr"/>
-      <c r="G101" s="16" t="inlineStr"/>
+      <c r="G101" s="15" t="inlineStr"/>
       <c r="H101" s="16" t="inlineStr"/>
-      <c r="I101" s="15" t="inlineStr"/>
+      <c r="I101" s="16" t="inlineStr"/>
       <c r="J101" s="15" t="inlineStr"/>
-      <c r="K101" s="17" t="inlineStr"/>
+      <c r="K101" s="15" t="inlineStr"/>
       <c r="L101" s="17" t="inlineStr"/>
       <c r="M101" s="17" t="inlineStr"/>
       <c r="N101" s="17" t="inlineStr"/>
@@ -5819,6 +5957,7 @@
       <c r="AI101" s="17" t="inlineStr"/>
       <c r="AJ101" s="17" t="inlineStr"/>
       <c r="AK101" s="17" t="inlineStr"/>
+      <c r="AL101" s="17" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" s="15" t="inlineStr"/>
@@ -5827,11 +5966,11 @@
       <c r="D102" s="15" t="inlineStr"/>
       <c r="E102" s="15" t="inlineStr"/>
       <c r="F102" s="15" t="inlineStr"/>
-      <c r="G102" s="16" t="inlineStr"/>
+      <c r="G102" s="15" t="inlineStr"/>
       <c r="H102" s="16" t="inlineStr"/>
-      <c r="I102" s="15" t="inlineStr"/>
+      <c r="I102" s="16" t="inlineStr"/>
       <c r="J102" s="15" t="inlineStr"/>
-      <c r="K102" s="17" t="inlineStr"/>
+      <c r="K102" s="15" t="inlineStr"/>
       <c r="L102" s="17" t="inlineStr"/>
       <c r="M102" s="17" t="inlineStr"/>
       <c r="N102" s="17" t="inlineStr"/>
@@ -5858,6 +5997,7 @@
       <c r="AI102" s="17" t="inlineStr"/>
       <c r="AJ102" s="17" t="inlineStr"/>
       <c r="AK102" s="17" t="inlineStr"/>
+      <c r="AL102" s="17" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" s="15" t="inlineStr"/>
@@ -5866,11 +6006,11 @@
       <c r="D103" s="15" t="inlineStr"/>
       <c r="E103" s="15" t="inlineStr"/>
       <c r="F103" s="15" t="inlineStr"/>
-      <c r="G103" s="16" t="inlineStr"/>
+      <c r="G103" s="15" t="inlineStr"/>
       <c r="H103" s="16" t="inlineStr"/>
-      <c r="I103" s="15" t="inlineStr"/>
+      <c r="I103" s="16" t="inlineStr"/>
       <c r="J103" s="15" t="inlineStr"/>
-      <c r="K103" s="17" t="inlineStr"/>
+      <c r="K103" s="15" t="inlineStr"/>
       <c r="L103" s="17" t="inlineStr"/>
       <c r="M103" s="17" t="inlineStr"/>
       <c r="N103" s="17" t="inlineStr"/>
@@ -5897,6 +6037,7 @@
       <c r="AI103" s="17" t="inlineStr"/>
       <c r="AJ103" s="17" t="inlineStr"/>
       <c r="AK103" s="17" t="inlineStr"/>
+      <c r="AL103" s="17" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" s="15" t="inlineStr"/>
@@ -5905,11 +6046,11 @@
       <c r="D104" s="15" t="inlineStr"/>
       <c r="E104" s="15" t="inlineStr"/>
       <c r="F104" s="15" t="inlineStr"/>
-      <c r="G104" s="16" t="inlineStr"/>
+      <c r="G104" s="15" t="inlineStr"/>
       <c r="H104" s="16" t="inlineStr"/>
-      <c r="I104" s="15" t="inlineStr"/>
+      <c r="I104" s="16" t="inlineStr"/>
       <c r="J104" s="15" t="inlineStr"/>
-      <c r="K104" s="17" t="inlineStr"/>
+      <c r="K104" s="15" t="inlineStr"/>
       <c r="L104" s="17" t="inlineStr"/>
       <c r="M104" s="17" t="inlineStr"/>
       <c r="N104" s="17" t="inlineStr"/>
@@ -5936,6 +6077,7 @@
       <c r="AI104" s="17" t="inlineStr"/>
       <c r="AJ104" s="17" t="inlineStr"/>
       <c r="AK104" s="17" t="inlineStr"/>
+      <c r="AL104" s="17" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" s="15" t="inlineStr"/>
@@ -5944,11 +6086,11 @@
       <c r="D105" s="15" t="inlineStr"/>
       <c r="E105" s="15" t="inlineStr"/>
       <c r="F105" s="15" t="inlineStr"/>
-      <c r="G105" s="16" t="inlineStr"/>
+      <c r="G105" s="15" t="inlineStr"/>
       <c r="H105" s="16" t="inlineStr"/>
-      <c r="I105" s="15" t="inlineStr"/>
+      <c r="I105" s="16" t="inlineStr"/>
       <c r="J105" s="15" t="inlineStr"/>
-      <c r="K105" s="17" t="inlineStr"/>
+      <c r="K105" s="15" t="inlineStr"/>
       <c r="L105" s="17" t="inlineStr"/>
       <c r="M105" s="17" t="inlineStr"/>
       <c r="N105" s="17" t="inlineStr"/>
@@ -5975,6 +6117,7 @@
       <c r="AI105" s="17" t="inlineStr"/>
       <c r="AJ105" s="17" t="inlineStr"/>
       <c r="AK105" s="17" t="inlineStr"/>
+      <c r="AL105" s="17" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" s="15" t="inlineStr"/>
@@ -5983,11 +6126,11 @@
       <c r="D106" s="15" t="inlineStr"/>
       <c r="E106" s="15" t="inlineStr"/>
       <c r="F106" s="15" t="inlineStr"/>
-      <c r="G106" s="16" t="inlineStr"/>
+      <c r="G106" s="15" t="inlineStr"/>
       <c r="H106" s="16" t="inlineStr"/>
-      <c r="I106" s="15" t="inlineStr"/>
+      <c r="I106" s="16" t="inlineStr"/>
       <c r="J106" s="15" t="inlineStr"/>
-      <c r="K106" s="17" t="inlineStr"/>
+      <c r="K106" s="15" t="inlineStr"/>
       <c r="L106" s="17" t="inlineStr"/>
       <c r="M106" s="17" t="inlineStr"/>
       <c r="N106" s="17" t="inlineStr"/>
@@ -6014,6 +6157,7 @@
       <c r="AI106" s="17" t="inlineStr"/>
       <c r="AJ106" s="17" t="inlineStr"/>
       <c r="AK106" s="17" t="inlineStr"/>
+      <c r="AL106" s="17" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" s="15" t="inlineStr"/>
@@ -6022,11 +6166,11 @@
       <c r="D107" s="15" t="inlineStr"/>
       <c r="E107" s="15" t="inlineStr"/>
       <c r="F107" s="15" t="inlineStr"/>
-      <c r="G107" s="16" t="inlineStr"/>
+      <c r="G107" s="15" t="inlineStr"/>
       <c r="H107" s="16" t="inlineStr"/>
-      <c r="I107" s="15" t="inlineStr"/>
+      <c r="I107" s="16" t="inlineStr"/>
       <c r="J107" s="15" t="inlineStr"/>
-      <c r="K107" s="17" t="inlineStr"/>
+      <c r="K107" s="15" t="inlineStr"/>
       <c r="L107" s="17" t="inlineStr"/>
       <c r="M107" s="17" t="inlineStr"/>
       <c r="N107" s="17" t="inlineStr"/>
@@ -6053,6 +6197,7 @@
       <c r="AI107" s="17" t="inlineStr"/>
       <c r="AJ107" s="17" t="inlineStr"/>
       <c r="AK107" s="17" t="inlineStr"/>
+      <c r="AL107" s="17" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" s="15" t="inlineStr"/>
@@ -6061,11 +6206,11 @@
       <c r="D108" s="15" t="inlineStr"/>
       <c r="E108" s="15" t="inlineStr"/>
       <c r="F108" s="15" t="inlineStr"/>
-      <c r="G108" s="16" t="inlineStr"/>
+      <c r="G108" s="15" t="inlineStr"/>
       <c r="H108" s="16" t="inlineStr"/>
-      <c r="I108" s="15" t="inlineStr"/>
+      <c r="I108" s="16" t="inlineStr"/>
       <c r="J108" s="15" t="inlineStr"/>
-      <c r="K108" s="17" t="inlineStr"/>
+      <c r="K108" s="15" t="inlineStr"/>
       <c r="L108" s="17" t="inlineStr"/>
       <c r="M108" s="17" t="inlineStr"/>
       <c r="N108" s="17" t="inlineStr"/>
@@ -6092,6 +6237,7 @@
       <c r="AI108" s="17" t="inlineStr"/>
       <c r="AJ108" s="17" t="inlineStr"/>
       <c r="AK108" s="17" t="inlineStr"/>
+      <c r="AL108" s="17" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" s="15" t="inlineStr"/>
@@ -6100,11 +6246,11 @@
       <c r="D109" s="15" t="inlineStr"/>
       <c r="E109" s="15" t="inlineStr"/>
       <c r="F109" s="15" t="inlineStr"/>
-      <c r="G109" s="16" t="inlineStr"/>
+      <c r="G109" s="15" t="inlineStr"/>
       <c r="H109" s="16" t="inlineStr"/>
-      <c r="I109" s="15" t="inlineStr"/>
+      <c r="I109" s="16" t="inlineStr"/>
       <c r="J109" s="15" t="inlineStr"/>
-      <c r="K109" s="17" t="inlineStr"/>
+      <c r="K109" s="15" t="inlineStr"/>
       <c r="L109" s="17" t="inlineStr"/>
       <c r="M109" s="17" t="inlineStr"/>
       <c r="N109" s="17" t="inlineStr"/>
@@ -6131,6 +6277,7 @@
       <c r="AI109" s="17" t="inlineStr"/>
       <c r="AJ109" s="17" t="inlineStr"/>
       <c r="AK109" s="17" t="inlineStr"/>
+      <c r="AL109" s="17" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" s="15" t="inlineStr"/>
@@ -6139,11 +6286,11 @@
       <c r="D110" s="15" t="inlineStr"/>
       <c r="E110" s="15" t="inlineStr"/>
       <c r="F110" s="15" t="inlineStr"/>
-      <c r="G110" s="16" t="inlineStr"/>
+      <c r="G110" s="15" t="inlineStr"/>
       <c r="H110" s="16" t="inlineStr"/>
-      <c r="I110" s="15" t="inlineStr"/>
+      <c r="I110" s="16" t="inlineStr"/>
       <c r="J110" s="15" t="inlineStr"/>
-      <c r="K110" s="17" t="inlineStr"/>
+      <c r="K110" s="15" t="inlineStr"/>
       <c r="L110" s="17" t="inlineStr"/>
       <c r="M110" s="17" t="inlineStr"/>
       <c r="N110" s="17" t="inlineStr"/>
@@ -6170,6 +6317,7 @@
       <c r="AI110" s="17" t="inlineStr"/>
       <c r="AJ110" s="17" t="inlineStr"/>
       <c r="AK110" s="17" t="inlineStr"/>
+      <c r="AL110" s="17" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" s="15" t="inlineStr"/>
@@ -6178,11 +6326,11 @@
       <c r="D111" s="15" t="inlineStr"/>
       <c r="E111" s="15" t="inlineStr"/>
       <c r="F111" s="15" t="inlineStr"/>
-      <c r="G111" s="16" t="inlineStr"/>
+      <c r="G111" s="15" t="inlineStr"/>
       <c r="H111" s="16" t="inlineStr"/>
-      <c r="I111" s="15" t="inlineStr"/>
+      <c r="I111" s="16" t="inlineStr"/>
       <c r="J111" s="15" t="inlineStr"/>
-      <c r="K111" s="17" t="inlineStr"/>
+      <c r="K111" s="15" t="inlineStr"/>
       <c r="L111" s="17" t="inlineStr"/>
       <c r="M111" s="17" t="inlineStr"/>
       <c r="N111" s="17" t="inlineStr"/>
@@ -6209,6 +6357,7 @@
       <c r="AI111" s="17" t="inlineStr"/>
       <c r="AJ111" s="17" t="inlineStr"/>
       <c r="AK111" s="17" t="inlineStr"/>
+      <c r="AL111" s="17" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" s="15" t="inlineStr"/>
@@ -6217,11 +6366,11 @@
       <c r="D112" s="15" t="inlineStr"/>
       <c r="E112" s="15" t="inlineStr"/>
       <c r="F112" s="15" t="inlineStr"/>
-      <c r="G112" s="16" t="inlineStr"/>
+      <c r="G112" s="15" t="inlineStr"/>
       <c r="H112" s="16" t="inlineStr"/>
-      <c r="I112" s="15" t="inlineStr"/>
+      <c r="I112" s="16" t="inlineStr"/>
       <c r="J112" s="15" t="inlineStr"/>
-      <c r="K112" s="17" t="inlineStr"/>
+      <c r="K112" s="15" t="inlineStr"/>
       <c r="L112" s="17" t="inlineStr"/>
       <c r="M112" s="17" t="inlineStr"/>
       <c r="N112" s="17" t="inlineStr"/>
@@ -6248,6 +6397,7 @@
       <c r="AI112" s="17" t="inlineStr"/>
       <c r="AJ112" s="17" t="inlineStr"/>
       <c r="AK112" s="17" t="inlineStr"/>
+      <c r="AL112" s="17" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" s="15" t="inlineStr"/>
@@ -6256,11 +6406,11 @@
       <c r="D113" s="15" t="inlineStr"/>
       <c r="E113" s="15" t="inlineStr"/>
       <c r="F113" s="15" t="inlineStr"/>
-      <c r="G113" s="16" t="inlineStr"/>
+      <c r="G113" s="15" t="inlineStr"/>
       <c r="H113" s="16" t="inlineStr"/>
-      <c r="I113" s="15" t="inlineStr"/>
+      <c r="I113" s="16" t="inlineStr"/>
       <c r="J113" s="15" t="inlineStr"/>
-      <c r="K113" s="17" t="inlineStr"/>
+      <c r="K113" s="15" t="inlineStr"/>
       <c r="L113" s="17" t="inlineStr"/>
       <c r="M113" s="17" t="inlineStr"/>
       <c r="N113" s="17" t="inlineStr"/>
@@ -6287,6 +6437,7 @@
       <c r="AI113" s="17" t="inlineStr"/>
       <c r="AJ113" s="17" t="inlineStr"/>
       <c r="AK113" s="17" t="inlineStr"/>
+      <c r="AL113" s="17" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" s="15" t="inlineStr"/>
@@ -6295,11 +6446,11 @@
       <c r="D114" s="15" t="inlineStr"/>
       <c r="E114" s="15" t="inlineStr"/>
       <c r="F114" s="15" t="inlineStr"/>
-      <c r="G114" s="16" t="inlineStr"/>
+      <c r="G114" s="15" t="inlineStr"/>
       <c r="H114" s="16" t="inlineStr"/>
-      <c r="I114" s="15" t="inlineStr"/>
+      <c r="I114" s="16" t="inlineStr"/>
       <c r="J114" s="15" t="inlineStr"/>
-      <c r="K114" s="17" t="inlineStr"/>
+      <c r="K114" s="15" t="inlineStr"/>
       <c r="L114" s="17" t="inlineStr"/>
       <c r="M114" s="17" t="inlineStr"/>
       <c r="N114" s="17" t="inlineStr"/>
@@ -6326,6 +6477,7 @@
       <c r="AI114" s="17" t="inlineStr"/>
       <c r="AJ114" s="17" t="inlineStr"/>
       <c r="AK114" s="17" t="inlineStr"/>
+      <c r="AL114" s="17" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" s="15" t="inlineStr"/>
@@ -6334,11 +6486,11 @@
       <c r="D115" s="15" t="inlineStr"/>
       <c r="E115" s="15" t="inlineStr"/>
       <c r="F115" s="15" t="inlineStr"/>
-      <c r="G115" s="16" t="inlineStr"/>
+      <c r="G115" s="15" t="inlineStr"/>
       <c r="H115" s="16" t="inlineStr"/>
-      <c r="I115" s="15" t="inlineStr"/>
+      <c r="I115" s="16" t="inlineStr"/>
       <c r="J115" s="15" t="inlineStr"/>
-      <c r="K115" s="17" t="inlineStr"/>
+      <c r="K115" s="15" t="inlineStr"/>
       <c r="L115" s="17" t="inlineStr"/>
       <c r="M115" s="17" t="inlineStr"/>
       <c r="N115" s="17" t="inlineStr"/>
@@ -6365,6 +6517,7 @@
       <c r="AI115" s="17" t="inlineStr"/>
       <c r="AJ115" s="17" t="inlineStr"/>
       <c r="AK115" s="17" t="inlineStr"/>
+      <c r="AL115" s="17" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" s="15" t="inlineStr"/>
@@ -6373,11 +6526,11 @@
       <c r="D116" s="15" t="inlineStr"/>
       <c r="E116" s="15" t="inlineStr"/>
       <c r="F116" s="15" t="inlineStr"/>
-      <c r="G116" s="16" t="inlineStr"/>
+      <c r="G116" s="15" t="inlineStr"/>
       <c r="H116" s="16" t="inlineStr"/>
-      <c r="I116" s="15" t="inlineStr"/>
+      <c r="I116" s="16" t="inlineStr"/>
       <c r="J116" s="15" t="inlineStr"/>
-      <c r="K116" s="17" t="inlineStr"/>
+      <c r="K116" s="15" t="inlineStr"/>
       <c r="L116" s="17" t="inlineStr"/>
       <c r="M116" s="17" t="inlineStr"/>
       <c r="N116" s="17" t="inlineStr"/>
@@ -6404,6 +6557,7 @@
       <c r="AI116" s="17" t="inlineStr"/>
       <c r="AJ116" s="17" t="inlineStr"/>
       <c r="AK116" s="17" t="inlineStr"/>
+      <c r="AL116" s="17" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" s="15" t="inlineStr"/>
@@ -6412,11 +6566,11 @@
       <c r="D117" s="15" t="inlineStr"/>
       <c r="E117" s="15" t="inlineStr"/>
       <c r="F117" s="15" t="inlineStr"/>
-      <c r="G117" s="16" t="inlineStr"/>
+      <c r="G117" s="15" t="inlineStr"/>
       <c r="H117" s="16" t="inlineStr"/>
-      <c r="I117" s="15" t="inlineStr"/>
+      <c r="I117" s="16" t="inlineStr"/>
       <c r="J117" s="15" t="inlineStr"/>
-      <c r="K117" s="17" t="inlineStr"/>
+      <c r="K117" s="15" t="inlineStr"/>
       <c r="L117" s="17" t="inlineStr"/>
       <c r="M117" s="17" t="inlineStr"/>
       <c r="N117" s="17" t="inlineStr"/>
@@ -6443,6 +6597,7 @@
       <c r="AI117" s="17" t="inlineStr"/>
       <c r="AJ117" s="17" t="inlineStr"/>
       <c r="AK117" s="17" t="inlineStr"/>
+      <c r="AL117" s="17" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" s="15" t="inlineStr"/>
@@ -6451,11 +6606,11 @@
       <c r="D118" s="15" t="inlineStr"/>
       <c r="E118" s="15" t="inlineStr"/>
       <c r="F118" s="15" t="inlineStr"/>
-      <c r="G118" s="16" t="inlineStr"/>
+      <c r="G118" s="15" t="inlineStr"/>
       <c r="H118" s="16" t="inlineStr"/>
-      <c r="I118" s="15" t="inlineStr"/>
+      <c r="I118" s="16" t="inlineStr"/>
       <c r="J118" s="15" t="inlineStr"/>
-      <c r="K118" s="17" t="inlineStr"/>
+      <c r="K118" s="15" t="inlineStr"/>
       <c r="L118" s="17" t="inlineStr"/>
       <c r="M118" s="17" t="inlineStr"/>
       <c r="N118" s="17" t="inlineStr"/>
@@ -6482,6 +6637,7 @@
       <c r="AI118" s="17" t="inlineStr"/>
       <c r="AJ118" s="17" t="inlineStr"/>
       <c r="AK118" s="17" t="inlineStr"/>
+      <c r="AL118" s="17" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" s="15" t="inlineStr"/>
@@ -6490,11 +6646,11 @@
       <c r="D119" s="15" t="inlineStr"/>
       <c r="E119" s="15" t="inlineStr"/>
       <c r="F119" s="15" t="inlineStr"/>
-      <c r="G119" s="16" t="inlineStr"/>
+      <c r="G119" s="15" t="inlineStr"/>
       <c r="H119" s="16" t="inlineStr"/>
-      <c r="I119" s="15" t="inlineStr"/>
+      <c r="I119" s="16" t="inlineStr"/>
       <c r="J119" s="15" t="inlineStr"/>
-      <c r="K119" s="17" t="inlineStr"/>
+      <c r="K119" s="15" t="inlineStr"/>
       <c r="L119" s="17" t="inlineStr"/>
       <c r="M119" s="17" t="inlineStr"/>
       <c r="N119" s="17" t="inlineStr"/>
@@ -6521,6 +6677,7 @@
       <c r="AI119" s="17" t="inlineStr"/>
       <c r="AJ119" s="17" t="inlineStr"/>
       <c r="AK119" s="17" t="inlineStr"/>
+      <c r="AL119" s="17" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" s="15" t="inlineStr"/>
@@ -6529,11 +6686,11 @@
       <c r="D120" s="15" t="inlineStr"/>
       <c r="E120" s="15" t="inlineStr"/>
       <c r="F120" s="15" t="inlineStr"/>
-      <c r="G120" s="16" t="inlineStr"/>
+      <c r="G120" s="15" t="inlineStr"/>
       <c r="H120" s="16" t="inlineStr"/>
-      <c r="I120" s="15" t="inlineStr"/>
+      <c r="I120" s="16" t="inlineStr"/>
       <c r="J120" s="15" t="inlineStr"/>
-      <c r="K120" s="17" t="inlineStr"/>
+      <c r="K120" s="15" t="inlineStr"/>
       <c r="L120" s="17" t="inlineStr"/>
       <c r="M120" s="17" t="inlineStr"/>
       <c r="N120" s="17" t="inlineStr"/>
@@ -6560,6 +6717,7 @@
       <c r="AI120" s="17" t="inlineStr"/>
       <c r="AJ120" s="17" t="inlineStr"/>
       <c r="AK120" s="17" t="inlineStr"/>
+      <c r="AL120" s="17" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" s="15" t="inlineStr"/>
@@ -6568,11 +6726,11 @@
       <c r="D121" s="15" t="inlineStr"/>
       <c r="E121" s="15" t="inlineStr"/>
       <c r="F121" s="15" t="inlineStr"/>
-      <c r="G121" s="16" t="inlineStr"/>
+      <c r="G121" s="15" t="inlineStr"/>
       <c r="H121" s="16" t="inlineStr"/>
-      <c r="I121" s="15" t="inlineStr"/>
+      <c r="I121" s="16" t="inlineStr"/>
       <c r="J121" s="15" t="inlineStr"/>
-      <c r="K121" s="17" t="inlineStr"/>
+      <c r="K121" s="15" t="inlineStr"/>
       <c r="L121" s="17" t="inlineStr"/>
       <c r="M121" s="17" t="inlineStr"/>
       <c r="N121" s="17" t="inlineStr"/>
@@ -6599,9 +6757,10 @@
       <c r="AI121" s="17" t="inlineStr"/>
       <c r="AJ121" s="17" t="inlineStr"/>
       <c r="AK121" s="17" t="inlineStr"/>
+      <c r="AL121" s="17" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:AK121"/>
+  <autoFilter ref="A1:AL121"/>
   <conditionalFormatting sqref="A2:A121">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$A2="Монетизация"</formula>
@@ -6619,21 +6778,24 @@
       <formula>$A2="Тарифы"</formula>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="A2:A121" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Неверное значение" error="Выберите значение из списка — так не будет разночтений." type="list">
       <formula1>=Справочник!$A$2:$A$6</formula1>
     </dataValidation>
     <dataValidation sqref="D2:D121" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Неверное значение" error="Выберите значение из списка — так не будет разночтений." type="list">
-      <formula1>=Справочник!$C$2:$C$4</formula1>
+      <formula1>=Справочник!$C$2:$C$3</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E121" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Неверное значение" error="Выберите значение из списка — так не будет разночтений." type="list">
       <formula1>=Справочник!$E$2:$E$38</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F121" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Неверное значение" error="Выберите значение из списка — так не будет разночтений." type="list">
-      <formula1>=Справочник!$G$2:$G$9</formula1>
+      <formula1>=Справочник!$G$2:$G$8</formula1>
     </dataValidation>
-    <dataValidation sqref="K2:AK121" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Неверное значение" error="Выберите значение из списка — так не будет разночтений." type="list">
-      <formula1>"1,2,3,4,5,отпуск"</formula1>
+    <dataValidation sqref="G2:G121" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Неверное значение" error="Выберите значение из списка — так не будет разночтений." type="list">
+      <formula1>"да"</formula1>
+    </dataValidation>
+    <dataValidation sqref="L2:AL121" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Неверное значение" error="Выберите значение из списка — так не будет разночтений." type="list">
+      <formula1>"1,2,3,4,5"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>